<commit_message>
Update Project Plan in Checklist
Updated Project Plan in Checklist
</commit_message>
<xml_diff>
--- a/ProjectManagement/Checklist.xlsx
+++ b/ProjectManagement/Checklist.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297DE719-9F34-4012-A557-27E115298C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82144DE2-E924-458C-91BE-F6B3C44B2CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -1755,32 +1755,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2007,6 +1986,27 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5183,6 +5183,241 @@
           <a:endParaRPr lang="en-IN" sz="1100"/>
         </a:p>
       </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>8962</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>62303</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>20665</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>167898</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="50" name="Rectangle 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5194E216-30DF-4684-B4CF-47EEDE2D442D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4542216" y="3456432"/>
+          <a:ext cx="621303" cy="105595"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>332154</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>77784</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>401624</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>162239</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="Rectangle 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F352768-30EA-4843-AF0F-5B899D49E341}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="4867248" y="3638126"/>
+          <a:ext cx="679504" cy="84455"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>604493</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>74182</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>95498</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>158637</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="52" name="Rectangle 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11D9E07F-3057-454E-8414-9C4613A7DB52}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="5136702" y="3828474"/>
+          <a:ext cx="708613" cy="84455"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>10159</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>75999</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>603884</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>160454</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="Rectangle 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F795F97-F99C-45D1-94EB-C3E534548A0A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="5763259" y="4007919"/>
+          <a:ext cx="593725" cy="84455"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>20730</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>73221</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>607854</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>157676</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="54" name="Rectangle 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{347CDCAA-3991-4290-B2BF-9C9775F76B27}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="5773433" y="4365424"/>
+          <a:ext cx="587124" cy="84455"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </xdr:spPr>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -13304,11 +13539,11 @@
       <c r="I6" s="9"/>
     </row>
     <row r="9" spans="1:9" ht="21">
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="142" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
+      <c r="C9" s="142"/>
+      <c r="D9" s="142"/>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
@@ -13330,12 +13565,12 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="21">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="142" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="64"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
+      <c r="B14" s="142"/>
+      <c r="C14" s="142"/>
+      <c r="D14" s="142"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15">
@@ -13344,7 +13579,7 @@
       <c r="B15" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="65" t="s">
+      <c r="C15" s="143" t="s">
         <v>125</v>
       </c>
     </row>
@@ -13356,7 +13591,7 @@
       <c r="B16" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="65"/>
+      <c r="C16" s="143"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17">
@@ -13366,7 +13601,7 @@
       <c r="B17" s="62" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="65"/>
+      <c r="C17" s="143"/>
     </row>
     <row r="18" spans="1:3">
       <c r="A18">
@@ -13376,7 +13611,7 @@
       <c r="B18" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="65"/>
+      <c r="C18" s="143"/>
     </row>
     <row r="19" spans="1:3">
       <c r="A19">
@@ -13386,7 +13621,7 @@
       <c r="B19" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="65"/>
+      <c r="C19" s="143"/>
     </row>
     <row r="20" spans="1:3">
       <c r="A20">
@@ -13396,7 +13631,7 @@
       <c r="B20" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="65"/>
+      <c r="C20" s="143"/>
     </row>
     <row r="21" spans="1:3">
       <c r="A21">
@@ -13406,7 +13641,7 @@
       <c r="B21" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="C21" s="65"/>
+      <c r="C21" s="143"/>
     </row>
     <row r="22" spans="1:3">
       <c r="A22">
@@ -13416,7 +13651,7 @@
       <c r="B22" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="65"/>
+      <c r="C22" s="143"/>
     </row>
     <row r="23" spans="1:3">
       <c r="A23">
@@ -13426,7 +13661,7 @@
       <c r="B23" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="65"/>
+      <c r="C23" s="143"/>
     </row>
     <row r="24" spans="1:3">
       <c r="A24">
@@ -13436,7 +13671,7 @@
       <c r="B24" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="65"/>
+      <c r="C24" s="143"/>
     </row>
     <row r="25" spans="1:3">
       <c r="A25">
@@ -13446,7 +13681,7 @@
       <c r="B25" s="62" t="s">
         <v>103</v>
       </c>
-      <c r="C25" s="65"/>
+      <c r="C25" s="143"/>
     </row>
     <row r="26" spans="1:3">
       <c r="A26">
@@ -13456,7 +13691,7 @@
       <c r="B26" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="66" t="s">
+      <c r="C26" s="144" t="s">
         <v>126</v>
       </c>
     </row>
@@ -13468,7 +13703,7 @@
       <c r="B27" t="s">
         <v>12</v>
       </c>
-      <c r="C27" s="66"/>
+      <c r="C27" s="144"/>
     </row>
     <row r="28" spans="1:3">
       <c r="A28">
@@ -13478,7 +13713,7 @@
       <c r="B28" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="66"/>
+      <c r="C28" s="144"/>
     </row>
     <row r="29" spans="1:3">
       <c r="A29">
@@ -13488,7 +13723,7 @@
       <c r="B29" t="s">
         <v>99</v>
       </c>
-      <c r="C29" s="66"/>
+      <c r="C29" s="144"/>
     </row>
     <row r="30" spans="1:3">
       <c r="A30">
@@ -13498,7 +13733,7 @@
       <c r="B30" t="s">
         <v>93</v>
       </c>
-      <c r="C30" s="66"/>
+      <c r="C30" s="144"/>
     </row>
     <row r="31" spans="1:3">
       <c r="A31">
@@ -13508,7 +13743,7 @@
       <c r="B31" t="s">
         <v>100</v>
       </c>
-      <c r="C31" s="66"/>
+      <c r="C31" s="144"/>
     </row>
     <row r="32" spans="1:3">
       <c r="A32">
@@ -13518,7 +13753,7 @@
       <c r="B32" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="66"/>
+      <c r="C32" s="144"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33">
@@ -13528,7 +13763,7 @@
       <c r="B33" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="66"/>
+      <c r="C33" s="144"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34">
@@ -13538,7 +13773,7 @@
       <c r="B34" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="65" t="s">
+      <c r="C34" s="143" t="s">
         <v>127</v>
       </c>
     </row>
@@ -13550,7 +13785,7 @@
       <c r="B35" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="65"/>
+      <c r="C35" s="143"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36">
@@ -13560,7 +13795,7 @@
       <c r="B36" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="C36" s="65"/>
+      <c r="C36" s="143"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37">
@@ -13570,15 +13805,15 @@
       <c r="B37" s="62" t="s">
         <v>102</v>
       </c>
-      <c r="C37" s="65"/>
+      <c r="C37" s="143"/>
     </row>
     <row r="38" spans="1:4" ht="21">
-      <c r="A38" s="64" t="s">
+      <c r="A38" s="142" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="64"/>
-      <c r="C38" s="64"/>
-      <c r="D38" s="64"/>
+      <c r="B38" s="142"/>
+      <c r="C38" s="142"/>
+      <c r="D38" s="142"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39">
@@ -13588,7 +13823,7 @@
       <c r="B39" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="66" t="s">
+      <c r="C39" s="144" t="s">
         <v>128</v>
       </c>
     </row>
@@ -13600,7 +13835,7 @@
       <c r="B40" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="66"/>
+      <c r="C40" s="144"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41">
@@ -13610,7 +13845,7 @@
       <c r="B41" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="66"/>
+      <c r="C41" s="144"/>
     </row>
     <row r="42" spans="1:4">
       <c r="A42">
@@ -13620,7 +13855,7 @@
       <c r="B42" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="66"/>
+      <c r="C42" s="144"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43">
@@ -13630,7 +13865,7 @@
       <c r="B43" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="66"/>
+      <c r="C43" s="144"/>
     </row>
     <row r="44" spans="1:4">
       <c r="A44">
@@ -13640,7 +13875,7 @@
       <c r="B44" t="s">
         <v>119</v>
       </c>
-      <c r="C44" s="66"/>
+      <c r="C44" s="144"/>
     </row>
     <row r="45" spans="1:4">
       <c r="A45">
@@ -13650,7 +13885,7 @@
       <c r="B45" t="s">
         <v>118</v>
       </c>
-      <c r="C45" s="66"/>
+      <c r="C45" s="144"/>
     </row>
     <row r="46" spans="1:4" ht="15" customHeight="1">
       <c r="A46">
@@ -13660,7 +13895,7 @@
       <c r="B46" s="62" t="s">
         <v>104</v>
       </c>
-      <c r="C46" s="67" t="s">
+      <c r="C46" s="145" t="s">
         <v>129</v>
       </c>
     </row>
@@ -13672,7 +13907,7 @@
       <c r="B47" s="62" t="s">
         <v>105</v>
       </c>
-      <c r="C47" s="67"/>
+      <c r="C47" s="145"/>
     </row>
     <row r="48" spans="1:4">
       <c r="A48">
@@ -13682,7 +13917,7 @@
       <c r="B48" s="62" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="67"/>
+      <c r="C48" s="145"/>
     </row>
     <row r="49" spans="1:3">
       <c r="A49">
@@ -13692,7 +13927,7 @@
       <c r="B49" s="62" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="67"/>
+      <c r="C49" s="145"/>
     </row>
     <row r="50" spans="1:3">
       <c r="A50">
@@ -13702,7 +13937,7 @@
       <c r="B50" t="s">
         <v>108</v>
       </c>
-      <c r="C50" s="68" t="s">
+      <c r="C50" s="146" t="s">
         <v>130</v>
       </c>
     </row>
@@ -13714,7 +13949,7 @@
       <c r="B51" t="s">
         <v>109</v>
       </c>
-      <c r="C51" s="68"/>
+      <c r="C51" s="146"/>
     </row>
     <row r="52" spans="1:3">
       <c r="A52">
@@ -13724,7 +13959,7 @@
       <c r="B52" t="s">
         <v>120</v>
       </c>
-      <c r="C52" s="68"/>
+      <c r="C52" s="146"/>
     </row>
     <row r="53" spans="1:3">
       <c r="A53">
@@ -13735,7 +13970,7 @@
         <f>[1]Report!$A$207</f>
         <v>Homework "Literature"</v>
       </c>
-      <c r="C53" s="67" t="s">
+      <c r="C53" s="145" t="s">
         <v>131</v>
       </c>
     </row>
@@ -13747,7 +13982,7 @@
       <c r="B54" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="C54" s="67"/>
+      <c r="C54" s="145"/>
     </row>
     <row r="55" spans="1:3">
       <c r="A55">
@@ -13757,7 +13992,7 @@
       <c r="B55" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="C55" s="67"/>
+      <c r="C55" s="145"/>
     </row>
     <row r="56" spans="1:3">
       <c r="A56">
@@ -13767,7 +14002,7 @@
       <c r="B56" t="s">
         <v>113</v>
       </c>
-      <c r="C56" s="68" t="s">
+      <c r="C56" s="146" t="s">
         <v>132</v>
       </c>
     </row>
@@ -13779,7 +14014,7 @@
       <c r="B57" t="s">
         <v>115</v>
       </c>
-      <c r="C57" s="68"/>
+      <c r="C57" s="146"/>
     </row>
     <row r="58" spans="1:3">
       <c r="A58">
@@ -13789,7 +14024,7 @@
       <c r="B58" t="s">
         <v>111</v>
       </c>
-      <c r="C58" s="68"/>
+      <c r="C58" s="146"/>
     </row>
     <row r="59" spans="1:3">
       <c r="A59">
@@ -13799,7 +14034,7 @@
       <c r="B59" t="s">
         <v>112</v>
       </c>
-      <c r="C59" s="68"/>
+      <c r="C59" s="146"/>
     </row>
     <row r="60" spans="1:3">
       <c r="A60">
@@ -13809,7 +14044,7 @@
       <c r="B60" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="C60" s="67" t="s">
+      <c r="C60" s="145" t="s">
         <v>133</v>
       </c>
     </row>
@@ -13821,7 +14056,7 @@
       <c r="B61" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="C61" s="67"/>
+      <c r="C61" s="145"/>
     </row>
     <row r="62" spans="1:3">
       <c r="A62">
@@ -13831,7 +14066,7 @@
       <c r="B62" s="62" t="s">
         <v>122</v>
       </c>
-      <c r="C62" s="67"/>
+      <c r="C62" s="145"/>
     </row>
     <row r="63" spans="1:3">
       <c r="A63">
@@ -13841,7 +14076,7 @@
       <c r="B63" t="s">
         <v>121</v>
       </c>
-      <c r="C63" s="68" t="s">
+      <c r="C63" s="146" t="s">
         <v>134</v>
       </c>
     </row>
@@ -13853,7 +14088,7 @@
       <c r="B64" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="C64" s="68"/>
+      <c r="C64" s="146"/>
     </row>
     <row r="65" spans="1:4">
       <c r="A65">
@@ -13863,15 +14098,15 @@
       <c r="B65" s="63" t="s">
         <v>124</v>
       </c>
-      <c r="C65" s="68"/>
+      <c r="C65" s="146"/>
     </row>
     <row r="66" spans="1:4" ht="21">
-      <c r="A66" s="64" t="s">
+      <c r="A66" s="142" t="s">
         <v>39</v>
       </c>
-      <c r="B66" s="64"/>
-      <c r="C66" s="64"/>
-      <c r="D66" s="64"/>
+      <c r="B66" s="142"/>
+      <c r="C66" s="142"/>
+      <c r="D66" s="142"/>
     </row>
     <row r="67" spans="1:4">
       <c r="A67">
@@ -14000,1872 +14235,1872 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="70"/>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="71"/>
-      <c r="AA1" s="71"/>
-      <c r="AB1" s="71"/>
-      <c r="AC1" s="71"/>
+      <c r="A1" s="64"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
+      <c r="O1" s="64"/>
+      <c r="P1" s="64"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
+      <c r="W1" s="65"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="65"/>
     </row>
     <row r="2" spans="1:29">
-      <c r="A2" s="70"/>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="71"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="71"/>
-      <c r="V2" s="71"/>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="71"/>
-      <c r="Z2" s="71"/>
-      <c r="AA2" s="71"/>
-      <c r="AB2" s="71"/>
-      <c r="AC2" s="71"/>
+      <c r="A2" s="64"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="64"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="65"/>
+      <c r="X2" s="65"/>
+      <c r="Y2" s="65"/>
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
     </row>
     <row r="3" spans="1:29">
-      <c r="A3" s="70"/>
-      <c r="B3" s="71"/>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="J3" s="70"/>
-      <c r="K3" s="70"/>
-      <c r="L3" s="70"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="71"/>
-      <c r="S3" s="71"/>
-      <c r="T3" s="71"/>
-      <c r="U3" s="71"/>
-      <c r="V3" s="71"/>
-      <c r="W3" s="71"/>
-      <c r="X3" s="71"/>
-      <c r="Y3" s="71"/>
-      <c r="Z3" s="71"/>
-      <c r="AA3" s="71"/>
-      <c r="AB3" s="71"/>
-      <c r="AC3" s="71"/>
+      <c r="A3" s="64"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="64"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="65"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="65"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="65"/>
+      <c r="AB3" s="65"/>
+      <c r="AC3" s="65"/>
     </row>
     <row r="4" spans="1:29">
-      <c r="A4" s="70"/>
-      <c r="B4" s="70"/>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="70"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="70"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="70"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="70"/>
-      <c r="S4" s="71"/>
-      <c r="T4" s="71"/>
-      <c r="U4" s="71"/>
-      <c r="V4" s="71"/>
-      <c r="W4" s="71"/>
-      <c r="X4" s="71"/>
-      <c r="Y4" s="71"/>
-      <c r="Z4" s="71"/>
-      <c r="AA4" s="71"/>
-      <c r="AB4" s="71"/>
-      <c r="AC4" s="71"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
+      <c r="R4" s="64"/>
+      <c r="S4" s="65"/>
+      <c r="T4" s="65"/>
+      <c r="U4" s="65"/>
+      <c r="V4" s="65"/>
+      <c r="W4" s="65"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="65"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="65"/>
     </row>
     <row r="5" spans="1:29">
-      <c r="A5" s="70"/>
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="70"/>
-      <c r="H5" s="70"/>
-      <c r="I5" s="70"/>
-      <c r="J5" s="70"/>
-      <c r="K5" s="70"/>
-      <c r="L5" s="70"/>
-      <c r="M5" s="70"/>
-      <c r="N5" s="70"/>
-      <c r="O5" s="70"/>
-      <c r="P5" s="70"/>
-      <c r="Q5" s="70"/>
-      <c r="R5" s="71"/>
-      <c r="S5" s="71"/>
-      <c r="T5" s="71"/>
-      <c r="U5" s="71"/>
-      <c r="V5" s="71"/>
-      <c r="W5" s="71"/>
-      <c r="X5" s="71"/>
-      <c r="Y5" s="71"/>
-      <c r="Z5" s="71"/>
-      <c r="AA5" s="71"/>
-      <c r="AB5" s="71"/>
-      <c r="AC5" s="71"/>
+      <c r="A5" s="64"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+      <c r="Q5" s="64"/>
+      <c r="R5" s="65"/>
+      <c r="S5" s="65"/>
+      <c r="T5" s="65"/>
+      <c r="U5" s="65"/>
+      <c r="V5" s="65"/>
+      <c r="W5" s="65"/>
+      <c r="X5" s="65"/>
+      <c r="Y5" s="65"/>
+      <c r="Z5" s="65"/>
+      <c r="AA5" s="65"/>
+      <c r="AB5" s="65"/>
+      <c r="AC5" s="65"/>
     </row>
     <row r="6" spans="1:29">
-      <c r="A6" s="70"/>
-      <c r="B6" s="71"/>
-      <c r="C6" s="71"/>
-      <c r="D6" s="71"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="70"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="70"/>
-      <c r="J6" s="70"/>
-      <c r="K6" s="70"/>
-      <c r="L6" s="70"/>
-      <c r="M6" s="70"/>
-      <c r="N6" s="70"/>
-      <c r="O6" s="70"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="70"/>
-      <c r="R6" s="71"/>
-      <c r="S6" s="71"/>
+      <c r="A6" s="64"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="64"/>
+      <c r="N6" s="64"/>
+      <c r="O6" s="64"/>
+      <c r="P6" s="64"/>
+      <c r="Q6" s="64"/>
+      <c r="R6" s="65"/>
+      <c r="S6" s="65"/>
       <c r="T6" t="s">
         <v>137</v>
       </c>
-      <c r="U6" s="71"/>
-      <c r="V6" s="71"/>
-      <c r="W6" s="71"/>
-      <c r="X6" s="71"/>
-      <c r="Y6" s="71"/>
-      <c r="Z6" s="71"/>
-      <c r="AA6" s="71"/>
-      <c r="AB6" s="71"/>
-      <c r="AC6" s="71"/>
+      <c r="U6" s="65"/>
+      <c r="V6" s="65"/>
+      <c r="W6" s="65"/>
+      <c r="X6" s="65"/>
+      <c r="Y6" s="65"/>
+      <c r="Z6" s="65"/>
+      <c r="AA6" s="65"/>
+      <c r="AB6" s="65"/>
+      <c r="AC6" s="65"/>
     </row>
     <row r="7" spans="1:29" ht="15.6">
-      <c r="A7" s="70"/>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="72"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="72"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="72"/>
-      <c r="K7" s="72"/>
-      <c r="L7" s="72"/>
-      <c r="M7" s="72"/>
-      <c r="N7" s="72"/>
-      <c r="O7" s="72"/>
-      <c r="P7" s="72"/>
-      <c r="Q7" s="72"/>
-      <c r="R7" s="71"/>
-      <c r="S7" s="71" t="s">
+      <c r="A7" s="64"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
+      <c r="J7" s="66"/>
+      <c r="K7" s="66"/>
+      <c r="L7" s="66"/>
+      <c r="M7" s="66"/>
+      <c r="N7" s="66"/>
+      <c r="O7" s="66"/>
+      <c r="P7" s="66"/>
+      <c r="Q7" s="66"/>
+      <c r="R7" s="65"/>
+      <c r="S7" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="T7" s="71" t="s">
+      <c r="T7" s="65" t="s">
         <v>138</v>
       </c>
-      <c r="U7" s="71"/>
-      <c r="V7" s="71"/>
-      <c r="W7" s="71"/>
-      <c r="X7" s="71"/>
-      <c r="Y7" s="71"/>
-      <c r="Z7" s="71"/>
-      <c r="AA7" s="71"/>
-      <c r="AB7" s="71"/>
-      <c r="AC7" s="71"/>
+      <c r="U7" s="65"/>
+      <c r="V7" s="65"/>
+      <c r="W7" s="65"/>
+      <c r="X7" s="65"/>
+      <c r="Y7" s="65"/>
+      <c r="Z7" s="65"/>
+      <c r="AA7" s="65"/>
+      <c r="AB7" s="65"/>
+      <c r="AC7" s="65"/>
     </row>
     <row r="8" spans="1:29" ht="17.399999999999999">
-      <c r="A8" s="70"/>
-      <c r="B8" s="70"/>
-      <c r="C8" s="70"/>
-      <c r="D8" s="70"/>
-      <c r="E8" s="73" t="s">
+      <c r="A8" s="64"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="147" t="s">
         <v>136</v>
       </c>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="M8" s="73"/>
-      <c r="N8" s="73"/>
-      <c r="O8" s="73"/>
-      <c r="P8" s="73"/>
-      <c r="Q8" s="73"/>
-      <c r="R8" s="71"/>
-      <c r="S8" s="71"/>
-      <c r="T8" s="71" t="s">
+      <c r="F8" s="147"/>
+      <c r="G8" s="147"/>
+      <c r="H8" s="147"/>
+      <c r="I8" s="147"/>
+      <c r="J8" s="147"/>
+      <c r="K8" s="147"/>
+      <c r="L8" s="147"/>
+      <c r="M8" s="147"/>
+      <c r="N8" s="147"/>
+      <c r="O8" s="147"/>
+      <c r="P8" s="147"/>
+      <c r="Q8" s="147"/>
+      <c r="R8" s="65"/>
+      <c r="S8" s="65"/>
+      <c r="T8" s="65" t="s">
         <v>139</v>
       </c>
-      <c r="U8" s="71"/>
-      <c r="V8" s="71"/>
-      <c r="W8" s="71"/>
-      <c r="X8" s="71"/>
-      <c r="Y8" s="71"/>
-      <c r="Z8" s="71"/>
-      <c r="AA8" s="71"/>
-      <c r="AB8" s="71"/>
-      <c r="AC8" s="71"/>
+      <c r="U8" s="65"/>
+      <c r="V8" s="65"/>
+      <c r="W8" s="65"/>
+      <c r="X8" s="65"/>
+      <c r="Y8" s="65"/>
+      <c r="Z8" s="65"/>
+      <c r="AA8" s="65"/>
+      <c r="AB8" s="65"/>
+      <c r="AC8" s="65"/>
     </row>
     <row r="9" spans="1:29" ht="15.6">
-      <c r="A9" s="70"/>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="72"/>
-      <c r="F9" s="72"/>
-      <c r="G9" s="72"/>
-      <c r="H9" s="72"/>
-      <c r="I9" s="72"/>
-      <c r="J9" s="72"/>
-      <c r="K9" s="72"/>
-      <c r="L9" s="72"/>
-      <c r="M9" s="72"/>
-      <c r="N9" s="72"/>
-      <c r="O9" s="72"/>
-      <c r="P9" s="72"/>
-      <c r="Q9" s="72"/>
-      <c r="R9" s="71"/>
-      <c r="S9" s="71"/>
-      <c r="T9" s="71"/>
-      <c r="U9" s="71"/>
-      <c r="V9" s="71"/>
-      <c r="W9" s="71"/>
-      <c r="X9" s="71"/>
-      <c r="Y9" s="71"/>
-      <c r="Z9" s="71"/>
-      <c r="AA9" s="71"/>
-      <c r="AB9" s="71"/>
-      <c r="AC9" s="71"/>
+      <c r="A9" s="64"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="66"/>
+      <c r="N9" s="66"/>
+      <c r="O9" s="66"/>
+      <c r="P9" s="66"/>
+      <c r="Q9" s="66"/>
+      <c r="R9" s="65"/>
+      <c r="S9" s="65"/>
+      <c r="T9" s="65"/>
+      <c r="U9" s="65"/>
+      <c r="V9" s="65"/>
+      <c r="W9" s="65"/>
+      <c r="X9" s="65"/>
+      <c r="Y9" s="65"/>
+      <c r="Z9" s="65"/>
+      <c r="AA9" s="65"/>
+      <c r="AB9" s="65"/>
+      <c r="AC9" s="65"/>
     </row>
     <row r="10" spans="1:29" ht="15" thickBot="1">
-      <c r="A10" s="70"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="70"/>
-      <c r="F10" s="70"/>
-      <c r="G10" s="70"/>
-      <c r="H10" s="70"/>
-      <c r="I10" s="70"/>
-      <c r="J10" s="70"/>
-      <c r="K10" s="70"/>
-      <c r="L10" s="70"/>
-      <c r="M10" s="70"/>
-      <c r="N10" s="70"/>
-      <c r="O10" s="70"/>
-      <c r="P10" s="70"/>
-      <c r="Q10" s="70"/>
-      <c r="R10" s="71"/>
-      <c r="S10" s="71"/>
-      <c r="T10" s="71"/>
-      <c r="U10" s="71"/>
-      <c r="V10" s="71"/>
-      <c r="W10" s="71"/>
-      <c r="X10" s="71"/>
-      <c r="Y10" s="71"/>
-      <c r="Z10" s="71"/>
-      <c r="AA10" s="71"/>
-      <c r="AB10" s="71"/>
-      <c r="AC10" s="71"/>
+      <c r="A10" s="64"/>
+      <c r="B10" s="65"/>
+      <c r="C10" s="65"/>
+      <c r="D10" s="65"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="64"/>
+      <c r="L10" s="64"/>
+      <c r="M10" s="64"/>
+      <c r="N10" s="64"/>
+      <c r="O10" s="64"/>
+      <c r="P10" s="64"/>
+      <c r="Q10" s="64"/>
+      <c r="R10" s="65"/>
+      <c r="S10" s="65"/>
+      <c r="T10" s="65"/>
+      <c r="U10" s="65"/>
+      <c r="V10" s="65"/>
+      <c r="W10" s="65"/>
+      <c r="X10" s="65"/>
+      <c r="Y10" s="65"/>
+      <c r="Z10" s="65"/>
+      <c r="AA10" s="65"/>
+      <c r="AB10" s="65"/>
+      <c r="AC10" s="65"/>
     </row>
     <row r="11" spans="1:29" ht="15" thickTop="1">
-      <c r="A11" s="74"/>
-      <c r="B11" s="75"/>
-      <c r="C11" s="76" t="s">
+      <c r="A11" s="67"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="D11" s="77">
+      <c r="D11" s="70">
         <v>40</v>
       </c>
-      <c r="E11" s="77">
+      <c r="E11" s="70">
         <v>41</v>
       </c>
-      <c r="F11" s="77">
+      <c r="F11" s="70">
         <v>42</v>
       </c>
-      <c r="G11" s="77">
+      <c r="G11" s="70">
         <v>43</v>
       </c>
-      <c r="H11" s="77">
+      <c r="H11" s="70">
         <v>44</v>
       </c>
-      <c r="I11" s="77">
+      <c r="I11" s="70">
         <v>45</v>
       </c>
-      <c r="J11" s="77">
+      <c r="J11" s="70">
         <v>46</v>
       </c>
-      <c r="K11" s="77">
+      <c r="K11" s="70">
         <v>47</v>
       </c>
-      <c r="L11" s="77">
+      <c r="L11" s="70">
         <v>48</v>
       </c>
-      <c r="M11" s="77">
+      <c r="M11" s="70">
         <v>49</v>
       </c>
-      <c r="N11" s="77">
+      <c r="N11" s="70">
         <v>50</v>
       </c>
-      <c r="O11" s="77">
+      <c r="O11" s="70">
         <v>51</v>
       </c>
-      <c r="P11" s="77">
+      <c r="P11" s="70">
         <v>52</v>
       </c>
-      <c r="Q11" s="77">
+      <c r="Q11" s="70">
         <v>1</v>
       </c>
-      <c r="R11" s="77">
+      <c r="R11" s="70">
         <v>2</v>
       </c>
-      <c r="S11" s="77">
+      <c r="S11" s="70">
         <v>3</v>
       </c>
-      <c r="T11" s="78">
+      <c r="T11" s="71">
         <v>4</v>
       </c>
-      <c r="U11" s="79">
+      <c r="U11" s="72">
         <v>5</v>
       </c>
-      <c r="V11" s="79">
+      <c r="V11" s="72">
         <v>6</v>
       </c>
-      <c r="W11" s="79">
+      <c r="W11" s="72">
         <v>7</v>
       </c>
-      <c r="X11" s="71"/>
-      <c r="Y11" s="71"/>
-      <c r="Z11" s="71"/>
-      <c r="AA11" s="71"/>
-      <c r="AB11" s="71"/>
-      <c r="AC11" s="71"/>
+      <c r="X11" s="65"/>
+      <c r="Y11" s="65"/>
+      <c r="Z11" s="65"/>
+      <c r="AA11" s="65"/>
+      <c r="AB11" s="65"/>
+      <c r="AC11" s="65"/>
     </row>
     <row r="12" spans="1:29">
-      <c r="A12" s="80"/>
-      <c r="B12" s="81"/>
-      <c r="C12" s="82" t="s">
+      <c r="A12" s="73"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="75" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="83">
+      <c r="D12" s="76">
         <v>1</v>
       </c>
-      <c r="E12" s="83">
+      <c r="E12" s="76">
         <v>2</v>
       </c>
-      <c r="F12" s="83">
+      <c r="F12" s="76">
         <v>3</v>
       </c>
-      <c r="G12" s="83">
+      <c r="G12" s="76">
         <v>4</v>
       </c>
-      <c r="H12" s="83">
+      <c r="H12" s="76">
         <v>5</v>
       </c>
-      <c r="I12" s="83">
+      <c r="I12" s="76">
         <v>6</v>
       </c>
-      <c r="J12" s="83">
+      <c r="J12" s="76">
         <v>7</v>
       </c>
-      <c r="K12" s="83">
+      <c r="K12" s="76">
         <v>8</v>
       </c>
-      <c r="L12" s="83">
+      <c r="L12" s="76">
         <v>9</v>
       </c>
-      <c r="M12" s="83">
+      <c r="M12" s="76">
         <v>10</v>
       </c>
-      <c r="N12" s="83">
+      <c r="N12" s="76">
         <v>11</v>
       </c>
-      <c r="O12" s="83">
+      <c r="O12" s="76">
         <v>12</v>
       </c>
-      <c r="P12" s="83">
+      <c r="P12" s="76">
         <v>13</v>
       </c>
-      <c r="Q12" s="83">
+      <c r="Q12" s="76">
         <v>14</v>
       </c>
-      <c r="R12" s="83">
+      <c r="R12" s="76">
         <v>15</v>
       </c>
-      <c r="S12" s="83">
+      <c r="S12" s="76">
         <v>16</v>
       </c>
-      <c r="T12" s="84">
+      <c r="T12" s="77">
         <v>17</v>
       </c>
-      <c r="U12" s="85">
+      <c r="U12" s="78">
         <v>18</v>
       </c>
-      <c r="V12" s="85">
+      <c r="V12" s="78">
         <v>19</v>
       </c>
-      <c r="W12" s="85">
+      <c r="W12" s="78">
         <v>20</v>
       </c>
-      <c r="X12" s="71"/>
-      <c r="Y12" s="71"/>
-      <c r="Z12" s="71"/>
-      <c r="AA12" s="71"/>
-      <c r="AB12" s="71"/>
-      <c r="AC12" s="71"/>
+      <c r="X12" s="65"/>
+      <c r="Y12" s="65"/>
+      <c r="Z12" s="65"/>
+      <c r="AA12" s="65"/>
+      <c r="AB12" s="65"/>
+      <c r="AC12" s="65"/>
     </row>
     <row r="13" spans="1:29" ht="15" thickBot="1">
-      <c r="A13" s="86" t="s">
+      <c r="A13" s="79" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="80" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="88" t="s">
+      <c r="C13" s="81" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="89"/>
-      <c r="E13" s="89"/>
-      <c r="F13" s="89"/>
-      <c r="G13" s="89"/>
-      <c r="H13" s="89"/>
-      <c r="I13" s="89"/>
-      <c r="J13" s="89"/>
-      <c r="K13" s="89"/>
-      <c r="L13" s="89"/>
-      <c r="M13" s="89"/>
-      <c r="N13" s="89"/>
-      <c r="O13" s="89"/>
-      <c r="P13" s="89"/>
-      <c r="Q13" s="89"/>
-      <c r="R13" s="89"/>
-      <c r="S13" s="89"/>
-      <c r="T13" s="90"/>
-      <c r="U13" s="91"/>
-      <c r="V13" s="91"/>
-      <c r="W13" s="91"/>
-      <c r="X13" s="71"/>
-      <c r="Y13" s="71"/>
-      <c r="Z13" s="71"/>
-      <c r="AA13" s="71"/>
-      <c r="AB13" s="71"/>
-      <c r="AC13" s="71"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="82"/>
+      <c r="L13" s="82"/>
+      <c r="M13" s="82"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="82"/>
+      <c r="Q13" s="82"/>
+      <c r="R13" s="82"/>
+      <c r="S13" s="82"/>
+      <c r="T13" s="83"/>
+      <c r="U13" s="84"/>
+      <c r="V13" s="84"/>
+      <c r="W13" s="84"/>
+      <c r="X13" s="65"/>
+      <c r="Y13" s="65"/>
+      <c r="Z13" s="65"/>
+      <c r="AA13" s="65"/>
+      <c r="AB13" s="65"/>
+      <c r="AC13" s="65"/>
     </row>
     <row r="14" spans="1:29">
-      <c r="A14" s="92">
+      <c r="A14" s="85">
         <v>1</v>
       </c>
-      <c r="B14" s="93" t="s">
+      <c r="B14" s="86" t="s">
         <v>140</v>
       </c>
-      <c r="C14" s="94">
+      <c r="C14" s="87">
         <v>2</v>
       </c>
-      <c r="D14" s="95"/>
-      <c r="E14" s="96"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="96"/>
-      <c r="H14" s="96"/>
-      <c r="I14" s="96"/>
-      <c r="J14" s="96"/>
-      <c r="K14" s="96"/>
-      <c r="L14" s="96"/>
-      <c r="M14" s="96"/>
-      <c r="N14" s="96"/>
-      <c r="O14" s="96"/>
-      <c r="P14" s="96"/>
-      <c r="Q14" s="96"/>
-      <c r="R14" s="96"/>
-      <c r="S14" s="96"/>
-      <c r="T14" s="96"/>
-      <c r="U14" s="96"/>
-      <c r="V14" s="97"/>
-      <c r="W14" s="97"/>
-      <c r="X14" s="71"/>
-      <c r="Y14" s="71"/>
-      <c r="Z14" s="71"/>
-      <c r="AA14" s="71"/>
-      <c r="AB14" s="71"/>
-      <c r="AC14" s="71"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="89"/>
+      <c r="G14" s="89"/>
+      <c r="H14" s="89"/>
+      <c r="I14" s="89"/>
+      <c r="J14" s="89"/>
+      <c r="K14" s="89"/>
+      <c r="L14" s="89"/>
+      <c r="M14" s="89"/>
+      <c r="N14" s="89"/>
+      <c r="O14" s="89"/>
+      <c r="P14" s="89"/>
+      <c r="Q14" s="89"/>
+      <c r="R14" s="89"/>
+      <c r="S14" s="89"/>
+      <c r="T14" s="89"/>
+      <c r="U14" s="89"/>
+      <c r="V14" s="90"/>
+      <c r="W14" s="90"/>
+      <c r="X14" s="65"/>
+      <c r="Y14" s="65"/>
+      <c r="Z14" s="65"/>
+      <c r="AA14" s="65"/>
+      <c r="AB14" s="65"/>
+      <c r="AC14" s="65"/>
     </row>
     <row r="15" spans="1:29">
-      <c r="A15" s="80">
+      <c r="A15" s="73">
         <v>2</v>
       </c>
-      <c r="B15" s="93" t="s">
+      <c r="B15" s="86" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="94">
+      <c r="C15" s="87">
         <v>1</v>
       </c>
-      <c r="D15" s="70"/>
-      <c r="E15" s="96"/>
-      <c r="F15" s="96"/>
-      <c r="G15" s="96"/>
-      <c r="H15" s="96"/>
-      <c r="I15" s="96"/>
-      <c r="J15" s="96"/>
-      <c r="K15" s="96"/>
-      <c r="L15" s="96"/>
-      <c r="M15" s="96"/>
-      <c r="N15" s="96"/>
-      <c r="O15" s="96"/>
-      <c r="P15" s="96"/>
-      <c r="Q15" s="96"/>
-      <c r="R15" s="96"/>
-      <c r="S15" s="96"/>
-      <c r="T15" s="96"/>
-      <c r="U15" s="96"/>
-      <c r="V15" s="97"/>
-      <c r="W15" s="97"/>
-      <c r="X15" s="71"/>
-      <c r="Y15" s="71"/>
-      <c r="Z15" s="71"/>
-      <c r="AA15" s="71"/>
-      <c r="AB15" s="71"/>
-      <c r="AC15" s="71"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+      <c r="K15" s="89"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="89"/>
+      <c r="N15" s="89"/>
+      <c r="O15" s="89"/>
+      <c r="P15" s="89"/>
+      <c r="Q15" s="89"/>
+      <c r="R15" s="89"/>
+      <c r="S15" s="89"/>
+      <c r="T15" s="89"/>
+      <c r="U15" s="89"/>
+      <c r="V15" s="90"/>
+      <c r="W15" s="90"/>
+      <c r="X15" s="65"/>
+      <c r="Y15" s="65"/>
+      <c r="Z15" s="65"/>
+      <c r="AA15" s="65"/>
+      <c r="AB15" s="65"/>
+      <c r="AC15" s="65"/>
     </row>
     <row r="16" spans="1:29">
-      <c r="A16" s="80">
+      <c r="A16" s="73">
         <v>3</v>
       </c>
-      <c r="B16" s="93" t="s">
+      <c r="B16" s="86" t="s">
         <v>142</v>
       </c>
-      <c r="C16" s="94">
+      <c r="C16" s="87">
         <v>2</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="E16" s="96"/>
-      <c r="F16" s="96"/>
-      <c r="G16" s="96"/>
-      <c r="H16" s="96"/>
-      <c r="I16" s="96"/>
-      <c r="J16" s="96"/>
-      <c r="K16" s="96"/>
-      <c r="L16" s="96"/>
-      <c r="M16" s="96"/>
-      <c r="N16" s="96"/>
-      <c r="O16" s="96"/>
-      <c r="P16" s="96"/>
-      <c r="Q16" s="96"/>
-      <c r="R16" s="96"/>
-      <c r="S16" s="96"/>
-      <c r="T16" s="96"/>
-      <c r="U16" s="96"/>
-      <c r="V16" s="97"/>
-      <c r="W16" s="97"/>
-      <c r="X16" s="71"/>
-      <c r="Y16" s="71"/>
-      <c r="Z16" s="71"/>
-      <c r="AA16" s="71"/>
-      <c r="AB16" s="71"/>
-      <c r="AC16" s="71"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="89"/>
+      <c r="F16" s="89"/>
+      <c r="G16" s="89"/>
+      <c r="H16" s="89"/>
+      <c r="I16" s="89"/>
+      <c r="J16" s="89"/>
+      <c r="K16" s="89"/>
+      <c r="L16" s="89"/>
+      <c r="M16" s="89"/>
+      <c r="N16" s="89"/>
+      <c r="O16" s="89"/>
+      <c r="P16" s="89"/>
+      <c r="Q16" s="89"/>
+      <c r="R16" s="89"/>
+      <c r="S16" s="89"/>
+      <c r="T16" s="89"/>
+      <c r="U16" s="89"/>
+      <c r="V16" s="90"/>
+      <c r="W16" s="90"/>
+      <c r="X16" s="65"/>
+      <c r="Y16" s="65"/>
+      <c r="Z16" s="65"/>
+      <c r="AA16" s="65"/>
+      <c r="AB16" s="65"/>
+      <c r="AC16" s="65"/>
     </row>
     <row r="17" spans="1:29">
-      <c r="A17" s="80">
+      <c r="A17" s="73">
         <v>4</v>
       </c>
-      <c r="B17" s="98" t="s">
+      <c r="B17" s="91" t="s">
         <v>143</v>
       </c>
-      <c r="C17" s="94">
+      <c r="C17" s="87">
         <v>2</v>
       </c>
-      <c r="D17" s="70"/>
-      <c r="E17" s="96"/>
-      <c r="F17" s="96"/>
-      <c r="G17" s="96"/>
-      <c r="H17" s="96"/>
-      <c r="I17" s="96"/>
-      <c r="J17" s="96"/>
-      <c r="K17" s="96"/>
-      <c r="L17" s="96"/>
-      <c r="M17" s="96"/>
-      <c r="N17" s="96"/>
-      <c r="O17" s="96"/>
-      <c r="P17" s="96"/>
-      <c r="Q17" s="96"/>
-      <c r="R17" s="96"/>
-      <c r="S17" s="96"/>
-      <c r="T17" s="96"/>
-      <c r="U17" s="96"/>
-      <c r="V17" s="97"/>
-      <c r="W17" s="97"/>
-      <c r="X17" s="71"/>
-      <c r="Y17" s="71"/>
-      <c r="Z17" s="71"/>
-      <c r="AA17" s="71"/>
-      <c r="AB17" s="71"/>
-      <c r="AC17" s="71"/>
+      <c r="D17" s="64"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
+      <c r="K17" s="89"/>
+      <c r="L17" s="89"/>
+      <c r="M17" s="89"/>
+      <c r="N17" s="89"/>
+      <c r="O17" s="89"/>
+      <c r="P17" s="89"/>
+      <c r="Q17" s="89"/>
+      <c r="R17" s="89"/>
+      <c r="S17" s="89"/>
+      <c r="T17" s="89"/>
+      <c r="U17" s="89"/>
+      <c r="V17" s="90"/>
+      <c r="W17" s="90"/>
+      <c r="X17" s="65"/>
+      <c r="Y17" s="65"/>
+      <c r="Z17" s="65"/>
+      <c r="AA17" s="65"/>
+      <c r="AB17" s="65"/>
+      <c r="AC17" s="65"/>
     </row>
     <row r="18" spans="1:29">
-      <c r="A18" s="80">
+      <c r="A18" s="73">
         <v>5</v>
       </c>
-      <c r="B18" s="99" t="s">
+      <c r="B18" s="92" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="100">
+      <c r="C18" s="93">
         <v>16</v>
       </c>
-      <c r="D18" s="101"/>
-      <c r="E18" s="102"/>
-      <c r="F18" s="103"/>
-      <c r="G18" s="103"/>
-      <c r="H18" s="103"/>
-      <c r="I18" s="103"/>
-      <c r="J18" s="103"/>
-      <c r="K18" s="103"/>
-      <c r="L18" s="103"/>
-      <c r="M18" s="103"/>
-      <c r="N18" s="103"/>
-      <c r="O18" s="103"/>
-      <c r="P18" s="103"/>
-      <c r="Q18" s="103"/>
-      <c r="R18" s="103"/>
-      <c r="S18" s="103"/>
-      <c r="T18" s="103"/>
-      <c r="U18" s="103"/>
-      <c r="V18" s="97"/>
-      <c r="W18" s="97"/>
-      <c r="X18" s="71"/>
-      <c r="Y18" s="71"/>
-      <c r="Z18" s="71"/>
-      <c r="AA18" s="71"/>
-      <c r="AB18" s="71"/>
-      <c r="AC18" s="71"/>
+      <c r="D18" s="94"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="96"/>
+      <c r="G18" s="96"/>
+      <c r="H18" s="96"/>
+      <c r="I18" s="96"/>
+      <c r="J18" s="96"/>
+      <c r="K18" s="96"/>
+      <c r="L18" s="96"/>
+      <c r="M18" s="96"/>
+      <c r="N18" s="96"/>
+      <c r="O18" s="96"/>
+      <c r="P18" s="96"/>
+      <c r="Q18" s="96"/>
+      <c r="R18" s="96"/>
+      <c r="S18" s="96"/>
+      <c r="T18" s="96"/>
+      <c r="U18" s="96"/>
+      <c r="V18" s="90"/>
+      <c r="W18" s="90"/>
+      <c r="X18" s="65"/>
+      <c r="Y18" s="65"/>
+      <c r="Z18" s="65"/>
+      <c r="AA18" s="65"/>
+      <c r="AB18" s="65"/>
+      <c r="AC18" s="65"/>
     </row>
     <row r="19" spans="1:29">
-      <c r="A19" s="80">
+      <c r="A19" s="73">
         <v>6</v>
       </c>
-      <c r="B19" s="108" t="s">
+      <c r="B19" s="101" t="s">
         <v>158</v>
       </c>
-      <c r="C19" s="94">
+      <c r="C19" s="87">
         <v>6</v>
       </c>
-      <c r="D19" s="101"/>
-      <c r="E19" s="104"/>
-      <c r="F19" s="97"/>
-      <c r="G19" s="97"/>
-      <c r="H19" s="97"/>
-      <c r="I19" s="97"/>
-      <c r="J19" s="97"/>
-      <c r="K19" s="97"/>
-      <c r="L19" s="97"/>
-      <c r="M19" s="97"/>
-      <c r="N19" s="97"/>
-      <c r="O19" s="97"/>
-      <c r="P19" s="97"/>
-      <c r="Q19" s="97"/>
-      <c r="R19" s="97"/>
-      <c r="S19" s="97"/>
-      <c r="T19" s="97"/>
-      <c r="U19" s="97"/>
-      <c r="V19" s="97"/>
-      <c r="W19" s="97"/>
-      <c r="X19" s="71"/>
-      <c r="Y19" s="71"/>
-      <c r="Z19" s="71"/>
-      <c r="AA19" s="71"/>
-      <c r="AB19" s="71"/>
-      <c r="AC19" s="71"/>
+      <c r="D19" s="94"/>
+      <c r="E19" s="97"/>
+      <c r="F19" s="90"/>
+      <c r="G19" s="90"/>
+      <c r="H19" s="90"/>
+      <c r="I19" s="90"/>
+      <c r="J19" s="90"/>
+      <c r="K19" s="90"/>
+      <c r="L19" s="90"/>
+      <c r="M19" s="90"/>
+      <c r="N19" s="90"/>
+      <c r="O19" s="90"/>
+      <c r="P19" s="90"/>
+      <c r="Q19" s="90"/>
+      <c r="R19" s="90"/>
+      <c r="S19" s="90"/>
+      <c r="T19" s="90"/>
+      <c r="U19" s="90"/>
+      <c r="V19" s="90"/>
+      <c r="W19" s="90"/>
+      <c r="X19" s="65"/>
+      <c r="Y19" s="65"/>
+      <c r="Z19" s="65"/>
+      <c r="AA19" s="65"/>
+      <c r="AB19" s="65"/>
+      <c r="AC19" s="65"/>
     </row>
     <row r="20" spans="1:29">
-      <c r="A20" s="80">
+      <c r="A20" s="73">
         <v>7</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="98" t="s">
         <v>144</v>
       </c>
-      <c r="C20" s="106">
+      <c r="C20" s="99">
         <v>5</v>
       </c>
-      <c r="D20" s="101"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="97"/>
-      <c r="G20" s="97"/>
-      <c r="H20" s="97"/>
-      <c r="I20" s="97"/>
-      <c r="J20" s="97"/>
-      <c r="K20" s="97"/>
-      <c r="L20" s="97"/>
-      <c r="M20" s="97"/>
-      <c r="N20" s="97"/>
-      <c r="O20" s="97"/>
-      <c r="P20" s="97"/>
-      <c r="Q20" s="97"/>
-      <c r="R20" s="97"/>
-      <c r="S20" s="97"/>
-      <c r="T20" s="97"/>
-      <c r="U20" s="97"/>
-      <c r="V20" s="97"/>
-      <c r="W20" s="97"/>
-      <c r="X20" s="71"/>
-      <c r="Y20" s="71"/>
-      <c r="Z20" s="71"/>
-      <c r="AA20" s="71"/>
-      <c r="AB20" s="71"/>
-      <c r="AC20" s="71"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="97"/>
+      <c r="F20" s="90"/>
+      <c r="G20" s="90"/>
+      <c r="H20" s="90"/>
+      <c r="I20" s="90"/>
+      <c r="J20" s="90"/>
+      <c r="K20" s="90"/>
+      <c r="L20" s="90"/>
+      <c r="M20" s="90"/>
+      <c r="N20" s="90"/>
+      <c r="O20" s="90"/>
+      <c r="P20" s="90"/>
+      <c r="Q20" s="90"/>
+      <c r="R20" s="90"/>
+      <c r="S20" s="90"/>
+      <c r="T20" s="90"/>
+      <c r="U20" s="90"/>
+      <c r="V20" s="90"/>
+      <c r="W20" s="90"/>
+      <c r="X20" s="65"/>
+      <c r="Y20" s="65"/>
+      <c r="Z20" s="65"/>
+      <c r="AA20" s="65"/>
+      <c r="AB20" s="65"/>
+      <c r="AC20" s="65"/>
     </row>
     <row r="21" spans="1:29">
-      <c r="A21" s="80">
+      <c r="A21" s="73">
         <v>8</v>
       </c>
-      <c r="B21" s="107" t="s">
+      <c r="B21" s="100" t="s">
         <v>145</v>
       </c>
-      <c r="C21" s="106">
+      <c r="C21" s="99">
         <v>5</v>
       </c>
-      <c r="D21" s="101"/>
-      <c r="E21" s="104"/>
-      <c r="F21" s="97"/>
-      <c r="G21" s="97"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="97"/>
-      <c r="K21" s="97"/>
-      <c r="L21" s="97"/>
-      <c r="M21" s="97"/>
-      <c r="N21" s="97"/>
-      <c r="O21" s="97"/>
-      <c r="P21" s="97"/>
-      <c r="Q21" s="97"/>
-      <c r="R21" s="97"/>
-      <c r="S21" s="97"/>
-      <c r="T21" s="97"/>
-      <c r="U21" s="97"/>
-      <c r="V21" s="97"/>
-      <c r="W21" s="97"/>
-      <c r="X21" s="71"/>
-      <c r="Y21" s="71"/>
-      <c r="Z21" s="71"/>
-      <c r="AA21" s="71"/>
-      <c r="AB21" s="71"/>
-      <c r="AC21" s="71"/>
+      <c r="D21" s="94"/>
+      <c r="E21" s="97"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
+      <c r="H21" s="90"/>
+      <c r="I21" s="90"/>
+      <c r="J21" s="90"/>
+      <c r="K21" s="90"/>
+      <c r="L21" s="90"/>
+      <c r="M21" s="90"/>
+      <c r="N21" s="90"/>
+      <c r="O21" s="90"/>
+      <c r="P21" s="90"/>
+      <c r="Q21" s="90"/>
+      <c r="R21" s="90"/>
+      <c r="S21" s="90"/>
+      <c r="T21" s="90"/>
+      <c r="U21" s="90"/>
+      <c r="V21" s="90"/>
+      <c r="W21" s="90"/>
+      <c r="X21" s="65"/>
+      <c r="Y21" s="65"/>
+      <c r="Z21" s="65"/>
+      <c r="AA21" s="65"/>
+      <c r="AB21" s="65"/>
+      <c r="AC21" s="65"/>
     </row>
     <row r="22" spans="1:29">
-      <c r="A22" s="80">
+      <c r="A22" s="73">
         <v>9</v>
       </c>
-      <c r="B22" s="108" t="s">
+      <c r="B22" s="105" t="s">
         <v>146</v>
       </c>
-      <c r="C22" s="106">
+      <c r="C22" s="99">
         <v>5</v>
       </c>
-      <c r="D22" s="101"/>
-      <c r="E22" s="104"/>
-      <c r="F22" s="97"/>
-      <c r="G22" s="97"/>
-      <c r="H22" s="97"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="97"/>
-      <c r="K22" s="97"/>
-      <c r="L22" s="97"/>
-      <c r="M22" s="97"/>
-      <c r="N22" s="97"/>
-      <c r="O22" s="97"/>
-      <c r="P22" s="97"/>
-      <c r="Q22" s="97"/>
-      <c r="R22" s="97"/>
-      <c r="S22" s="97"/>
-      <c r="T22" s="97"/>
-      <c r="U22" s="97"/>
-      <c r="V22" s="97"/>
-      <c r="W22" s="97"/>
-      <c r="X22" s="71"/>
-      <c r="Y22" s="71"/>
-      <c r="Z22" s="71"/>
-      <c r="AA22" s="71"/>
-      <c r="AB22" s="71"/>
-      <c r="AC22" s="71"/>
+      <c r="D22" s="94"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="90"/>
+      <c r="G22" s="90"/>
+      <c r="H22" s="90"/>
+      <c r="I22" s="90"/>
+      <c r="J22" s="90"/>
+      <c r="K22" s="90"/>
+      <c r="L22" s="90"/>
+      <c r="M22" s="90"/>
+      <c r="N22" s="90"/>
+      <c r="O22" s="90"/>
+      <c r="P22" s="90"/>
+      <c r="Q22" s="90"/>
+      <c r="R22" s="90"/>
+      <c r="S22" s="90"/>
+      <c r="T22" s="90"/>
+      <c r="U22" s="90"/>
+      <c r="V22" s="90"/>
+      <c r="W22" s="90"/>
+      <c r="X22" s="65"/>
+      <c r="Y22" s="65"/>
+      <c r="Z22" s="65"/>
+      <c r="AA22" s="65"/>
+      <c r="AB22" s="65"/>
+      <c r="AC22" s="65"/>
     </row>
     <row r="23" spans="1:29">
-      <c r="A23" s="80">
+      <c r="A23" s="73">
         <v>10</v>
       </c>
-      <c r="B23" s="107" t="s">
+      <c r="B23" s="100" t="s">
         <v>147</v>
       </c>
-      <c r="C23" s="106">
+      <c r="C23" s="99">
         <v>5</v>
       </c>
-      <c r="D23" s="101"/>
-      <c r="E23" s="104"/>
-      <c r="F23" s="97"/>
-      <c r="G23" s="97"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="97"/>
-      <c r="K23" s="97"/>
-      <c r="L23" s="97"/>
-      <c r="M23" s="97"/>
-      <c r="N23" s="97"/>
-      <c r="O23" s="97"/>
-      <c r="P23" s="97"/>
-      <c r="Q23" s="97"/>
-      <c r="R23" s="97"/>
-      <c r="S23" s="97"/>
-      <c r="T23" s="97"/>
-      <c r="U23" s="97"/>
-      <c r="V23" s="97"/>
-      <c r="W23" s="97"/>
-      <c r="X23" s="71"/>
-      <c r="Y23" s="71"/>
-      <c r="Z23" s="71"/>
-      <c r="AA23" s="71"/>
-      <c r="AB23" s="71"/>
-      <c r="AC23" s="71"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="97"/>
+      <c r="F23" s="90"/>
+      <c r="G23" s="90"/>
+      <c r="H23" s="90"/>
+      <c r="I23" s="90"/>
+      <c r="J23" s="90"/>
+      <c r="K23" s="90"/>
+      <c r="L23" s="90"/>
+      <c r="M23" s="90"/>
+      <c r="N23" s="90"/>
+      <c r="O23" s="90"/>
+      <c r="P23" s="90"/>
+      <c r="Q23" s="90"/>
+      <c r="R23" s="90"/>
+      <c r="S23" s="90"/>
+      <c r="T23" s="90"/>
+      <c r="U23" s="90"/>
+      <c r="V23" s="90"/>
+      <c r="W23" s="90"/>
+      <c r="X23" s="65"/>
+      <c r="Y23" s="65"/>
+      <c r="Z23" s="65"/>
+      <c r="AA23" s="65"/>
+      <c r="AB23" s="65"/>
+      <c r="AC23" s="65"/>
     </row>
     <row r="24" spans="1:29">
-      <c r="A24" s="80">
+      <c r="A24" s="73">
         <v>11</v>
       </c>
-      <c r="B24" s="109" t="s">
+      <c r="B24" s="102" t="s">
         <v>175</v>
       </c>
-      <c r="C24" s="106">
+      <c r="C24" s="99">
         <v>5</v>
       </c>
-      <c r="D24" s="101"/>
-      <c r="E24" s="104"/>
-      <c r="F24" s="97"/>
-      <c r="G24" s="97"/>
-      <c r="H24" s="97"/>
-      <c r="I24" s="97"/>
-      <c r="J24" s="97"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="97"/>
-      <c r="N24" s="97"/>
-      <c r="O24" s="97"/>
-      <c r="P24" s="97"/>
-      <c r="Q24" s="97"/>
-      <c r="R24" s="97"/>
-      <c r="S24" s="97"/>
-      <c r="T24" s="97"/>
-      <c r="U24" s="97"/>
-      <c r="V24" s="97"/>
-      <c r="W24" s="97"/>
-      <c r="X24" s="71"/>
-      <c r="Y24" s="71"/>
-      <c r="Z24" s="71"/>
-      <c r="AA24" s="71"/>
-      <c r="AB24" s="71"/>
-      <c r="AC24" s="71"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="97"/>
+      <c r="F24" s="90"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="90"/>
+      <c r="I24" s="90"/>
+      <c r="J24" s="90"/>
+      <c r="K24" s="90"/>
+      <c r="L24" s="90"/>
+      <c r="M24" s="90"/>
+      <c r="N24" s="90"/>
+      <c r="O24" s="90"/>
+      <c r="P24" s="90"/>
+      <c r="Q24" s="90"/>
+      <c r="R24" s="90"/>
+      <c r="S24" s="90"/>
+      <c r="T24" s="90"/>
+      <c r="U24" s="90"/>
+      <c r="V24" s="90"/>
+      <c r="W24" s="90"/>
+      <c r="X24" s="65"/>
+      <c r="Y24" s="65"/>
+      <c r="Z24" s="65"/>
+      <c r="AA24" s="65"/>
+      <c r="AB24" s="65"/>
+      <c r="AC24" s="65"/>
     </row>
     <row r="25" spans="1:29">
-      <c r="A25" s="80">
+      <c r="A25" s="73">
         <v>12</v>
       </c>
-      <c r="B25" s="109" t="s">
+      <c r="B25" s="102" t="s">
         <v>148</v>
       </c>
-      <c r="C25" s="106">
+      <c r="C25" s="99">
         <v>7</v>
       </c>
-      <c r="D25" s="101"/>
-      <c r="E25" s="104"/>
-      <c r="F25" s="97"/>
-      <c r="G25" s="97"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="97"/>
-      <c r="L25" s="97"/>
-      <c r="M25" s="97"/>
-      <c r="N25" s="97"/>
-      <c r="O25" s="97"/>
-      <c r="P25" s="97"/>
-      <c r="Q25" s="97"/>
-      <c r="R25" s="97"/>
-      <c r="S25" s="97"/>
-      <c r="T25" s="97"/>
-      <c r="U25" s="97"/>
-      <c r="V25" s="97"/>
-      <c r="W25" s="97"/>
-      <c r="X25" s="71"/>
-      <c r="Y25" s="71"/>
-      <c r="Z25" s="71"/>
-      <c r="AA25" s="71"/>
-      <c r="AB25" s="71"/>
-      <c r="AC25" s="71"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="97"/>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
+      <c r="J25" s="90"/>
+      <c r="K25" s="90"/>
+      <c r="L25" s="90"/>
+      <c r="M25" s="90"/>
+      <c r="N25" s="90"/>
+      <c r="O25" s="90"/>
+      <c r="P25" s="90"/>
+      <c r="Q25" s="90"/>
+      <c r="R25" s="90"/>
+      <c r="S25" s="90"/>
+      <c r="T25" s="90"/>
+      <c r="U25" s="90"/>
+      <c r="V25" s="90"/>
+      <c r="W25" s="90"/>
+      <c r="X25" s="65"/>
+      <c r="Y25" s="65"/>
+      <c r="Z25" s="65"/>
+      <c r="AA25" s="65"/>
+      <c r="AB25" s="65"/>
+      <c r="AC25" s="65"/>
     </row>
     <row r="26" spans="1:29">
-      <c r="A26" s="80">
+      <c r="A26" s="73">
         <v>13</v>
       </c>
-      <c r="B26" s="110" t="s">
+      <c r="B26" s="103" t="s">
         <v>149</v>
       </c>
-      <c r="C26" s="106">
+      <c r="C26" s="99">
         <v>5</v>
       </c>
-      <c r="D26" s="101"/>
-      <c r="E26" s="104"/>
-      <c r="F26" s="97"/>
-      <c r="G26" s="97"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="97"/>
-      <c r="L26" s="97"/>
-      <c r="M26" s="97"/>
-      <c r="N26" s="97"/>
-      <c r="O26" s="97"/>
-      <c r="P26" s="97"/>
-      <c r="Q26" s="97"/>
-      <c r="R26" s="97"/>
-      <c r="S26" s="97"/>
-      <c r="T26" s="97"/>
-      <c r="U26" s="97"/>
-      <c r="V26" s="97"/>
-      <c r="W26" s="97"/>
-      <c r="X26" s="71"/>
-      <c r="Y26" s="71"/>
-      <c r="Z26" s="71"/>
-      <c r="AA26" s="71"/>
-      <c r="AB26" s="71"/>
-      <c r="AC26" s="71"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="97"/>
+      <c r="F26" s="90"/>
+      <c r="G26" s="90"/>
+      <c r="H26" s="90"/>
+      <c r="I26" s="90"/>
+      <c r="J26" s="90"/>
+      <c r="K26" s="90"/>
+      <c r="L26" s="90"/>
+      <c r="M26" s="90"/>
+      <c r="N26" s="90"/>
+      <c r="O26" s="90"/>
+      <c r="P26" s="90"/>
+      <c r="Q26" s="90"/>
+      <c r="R26" s="90"/>
+      <c r="S26" s="90"/>
+      <c r="T26" s="90"/>
+      <c r="U26" s="90"/>
+      <c r="V26" s="90"/>
+      <c r="W26" s="90"/>
+      <c r="X26" s="65"/>
+      <c r="Y26" s="65"/>
+      <c r="Z26" s="65"/>
+      <c r="AA26" s="65"/>
+      <c r="AB26" s="65"/>
+      <c r="AC26" s="65"/>
     </row>
     <row r="27" spans="1:29">
-      <c r="A27" s="80">
+      <c r="A27" s="73">
         <v>14</v>
       </c>
-      <c r="B27" s="111" t="s">
+      <c r="B27" s="104" t="s">
         <v>150</v>
       </c>
-      <c r="C27" s="106">
+      <c r="C27" s="99">
         <v>6</v>
       </c>
-      <c r="D27" s="101"/>
-      <c r="E27" s="104"/>
-      <c r="F27" s="97"/>
-      <c r="G27" s="97"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="97"/>
-      <c r="K27" s="97"/>
-      <c r="L27" s="97"/>
-      <c r="M27" s="97"/>
-      <c r="N27" s="97"/>
-      <c r="O27" s="97"/>
-      <c r="P27" s="97"/>
-      <c r="Q27" s="97"/>
-      <c r="R27" s="97"/>
-      <c r="S27" s="97"/>
-      <c r="T27" s="97"/>
-      <c r="U27" s="97"/>
-      <c r="V27" s="97"/>
-      <c r="W27" s="97"/>
-      <c r="X27" s="71"/>
-      <c r="Y27" s="71"/>
-      <c r="Z27" s="71"/>
-      <c r="AA27" s="71"/>
-      <c r="AB27" s="71"/>
-      <c r="AC27" s="71"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="97"/>
+      <c r="F27" s="90"/>
+      <c r="G27" s="90"/>
+      <c r="H27" s="90"/>
+      <c r="I27" s="90"/>
+      <c r="J27" s="90"/>
+      <c r="K27" s="90"/>
+      <c r="L27" s="90"/>
+      <c r="M27" s="90"/>
+      <c r="N27" s="90"/>
+      <c r="O27" s="90"/>
+      <c r="P27" s="90"/>
+      <c r="Q27" s="90"/>
+      <c r="R27" s="90"/>
+      <c r="S27" s="90"/>
+      <c r="T27" s="90"/>
+      <c r="U27" s="90"/>
+      <c r="V27" s="90"/>
+      <c r="W27" s="90"/>
+      <c r="X27" s="65"/>
+      <c r="Y27" s="65"/>
+      <c r="Z27" s="65"/>
+      <c r="AA27" s="65"/>
+      <c r="AB27" s="65"/>
+      <c r="AC27" s="65"/>
     </row>
     <row r="28" spans="1:29">
-      <c r="A28" s="80">
+      <c r="A28" s="73">
         <v>15</v>
       </c>
-      <c r="B28" s="112" t="s">
+      <c r="B28" s="105" t="s">
         <v>151</v>
       </c>
-      <c r="C28" s="106">
+      <c r="C28" s="99">
         <v>6</v>
       </c>
-      <c r="D28" s="101"/>
-      <c r="E28" s="104"/>
-      <c r="F28" s="97"/>
-      <c r="G28" s="97"/>
-      <c r="H28" s="97"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="97"/>
-      <c r="K28" s="97"/>
-      <c r="L28" s="97"/>
-      <c r="M28" s="97"/>
-      <c r="N28" s="97"/>
-      <c r="O28" s="97"/>
-      <c r="P28" s="97"/>
-      <c r="Q28" s="97"/>
-      <c r="R28" s="97"/>
-      <c r="S28" s="97"/>
-      <c r="T28" s="97"/>
-      <c r="U28" s="97"/>
-      <c r="V28" s="97"/>
-      <c r="W28" s="97"/>
-      <c r="X28" s="71"/>
-      <c r="Y28" s="71"/>
-      <c r="Z28" s="71"/>
-      <c r="AA28" s="71"/>
-      <c r="AB28" s="71"/>
-      <c r="AC28" s="71"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="90"/>
+      <c r="G28" s="90"/>
+      <c r="H28" s="90"/>
+      <c r="I28" s="90"/>
+      <c r="J28" s="90"/>
+      <c r="K28" s="90"/>
+      <c r="L28" s="90"/>
+      <c r="M28" s="90"/>
+      <c r="N28" s="90"/>
+      <c r="O28" s="90"/>
+      <c r="P28" s="90"/>
+      <c r="Q28" s="90"/>
+      <c r="R28" s="90"/>
+      <c r="S28" s="90"/>
+      <c r="T28" s="90"/>
+      <c r="U28" s="90"/>
+      <c r="V28" s="90"/>
+      <c r="W28" s="90"/>
+      <c r="X28" s="65"/>
+      <c r="Y28" s="65"/>
+      <c r="Z28" s="65"/>
+      <c r="AA28" s="65"/>
+      <c r="AB28" s="65"/>
+      <c r="AC28" s="65"/>
     </row>
     <row r="29" spans="1:29">
-      <c r="A29" s="80">
+      <c r="A29" s="73">
         <v>16</v>
       </c>
-      <c r="B29" s="105" t="s">
+      <c r="B29" s="98" t="s">
         <v>152</v>
       </c>
-      <c r="C29" s="106">
+      <c r="C29" s="99">
         <v>6</v>
       </c>
-      <c r="D29" s="101"/>
-      <c r="E29" s="104"/>
-      <c r="F29" s="97"/>
-      <c r="G29" s="97"/>
-      <c r="H29" s="97"/>
-      <c r="I29" s="97"/>
-      <c r="J29" s="97"/>
-      <c r="K29" s="97"/>
-      <c r="L29" s="97"/>
-      <c r="M29" s="97"/>
-      <c r="N29" s="97"/>
-      <c r="O29" s="97"/>
-      <c r="P29" s="97"/>
-      <c r="Q29" s="97"/>
-      <c r="R29" s="97"/>
-      <c r="S29" s="97"/>
-      <c r="T29" s="97"/>
-      <c r="U29" s="97"/>
-      <c r="V29" s="97"/>
-      <c r="W29" s="97"/>
-      <c r="X29" s="71"/>
-      <c r="Y29" s="71"/>
-      <c r="Z29" s="71"/>
-      <c r="AA29" s="71"/>
-      <c r="AB29" s="71"/>
-      <c r="AC29" s="71"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="97"/>
+      <c r="F29" s="90"/>
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="I29" s="90"/>
+      <c r="J29" s="90"/>
+      <c r="K29" s="90"/>
+      <c r="L29" s="90"/>
+      <c r="M29" s="90"/>
+      <c r="N29" s="90"/>
+      <c r="O29" s="90"/>
+      <c r="P29" s="90"/>
+      <c r="Q29" s="90"/>
+      <c r="R29" s="90"/>
+      <c r="S29" s="90"/>
+      <c r="T29" s="90"/>
+      <c r="U29" s="90"/>
+      <c r="V29" s="90"/>
+      <c r="W29" s="90"/>
+      <c r="X29" s="65"/>
+      <c r="Y29" s="65"/>
+      <c r="Z29" s="65"/>
+      <c r="AA29" s="65"/>
+      <c r="AB29" s="65"/>
+      <c r="AC29" s="65"/>
     </row>
     <row r="30" spans="1:29">
-      <c r="A30" s="80">
+      <c r="A30" s="73">
         <v>17</v>
       </c>
-      <c r="B30" s="111" t="s">
+      <c r="B30" s="104" t="s">
         <v>153</v>
       </c>
-      <c r="C30" s="106">
+      <c r="C30" s="99">
         <v>7</v>
       </c>
-      <c r="D30" s="101"/>
-      <c r="E30" s="104"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="97"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
-      <c r="J30" s="97"/>
-      <c r="K30" s="97"/>
-      <c r="L30" s="97"/>
-      <c r="M30" s="97"/>
-      <c r="N30" s="97"/>
-      <c r="O30" s="97"/>
-      <c r="P30" s="97"/>
-      <c r="Q30" s="97"/>
-      <c r="R30" s="97"/>
-      <c r="S30" s="97"/>
-      <c r="T30" s="97"/>
-      <c r="U30" s="97"/>
-      <c r="V30" s="97"/>
-      <c r="W30" s="97"/>
-      <c r="X30" s="71"/>
-      <c r="Y30" s="71"/>
-      <c r="Z30" s="71"/>
-      <c r="AA30" s="71"/>
-      <c r="AB30" s="71"/>
-      <c r="AC30" s="71"/>
+      <c r="D30" s="94"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="90"/>
+      <c r="G30" s="90"/>
+      <c r="H30" s="90"/>
+      <c r="I30" s="90"/>
+      <c r="J30" s="90"/>
+      <c r="K30" s="90"/>
+      <c r="L30" s="90"/>
+      <c r="M30" s="90"/>
+      <c r="N30" s="90"/>
+      <c r="O30" s="90"/>
+      <c r="P30" s="90"/>
+      <c r="Q30" s="90"/>
+      <c r="R30" s="90"/>
+      <c r="S30" s="90"/>
+      <c r="T30" s="90"/>
+      <c r="U30" s="90"/>
+      <c r="V30" s="90"/>
+      <c r="W30" s="90"/>
+      <c r="X30" s="65"/>
+      <c r="Y30" s="65"/>
+      <c r="Z30" s="65"/>
+      <c r="AA30" s="65"/>
+      <c r="AB30" s="65"/>
+      <c r="AC30" s="65"/>
     </row>
     <row r="31" spans="1:29">
-      <c r="A31" s="80">
+      <c r="A31" s="73">
         <v>18</v>
       </c>
-      <c r="B31" s="112" t="s">
+      <c r="B31" s="105" t="s">
         <v>154</v>
       </c>
-      <c r="C31" s="106">
+      <c r="C31" s="99">
         <v>7</v>
       </c>
-      <c r="D31" s="101"/>
-      <c r="E31" s="104"/>
-      <c r="F31" s="97"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="97"/>
-      <c r="J31" s="97"/>
-      <c r="K31" s="97"/>
-      <c r="L31" s="97"/>
-      <c r="M31" s="97"/>
-      <c r="N31" s="97"/>
-      <c r="O31" s="97"/>
-      <c r="P31" s="97"/>
-      <c r="Q31" s="97"/>
-      <c r="R31" s="97"/>
-      <c r="S31" s="97"/>
-      <c r="T31" s="97"/>
-      <c r="U31" s="97"/>
-      <c r="V31" s="97"/>
-      <c r="W31" s="97"/>
-      <c r="X31" s="71"/>
-      <c r="Y31" s="71"/>
-      <c r="Z31" s="71"/>
-      <c r="AA31" s="71"/>
-      <c r="AB31" s="71"/>
-      <c r="AC31" s="71"/>
+      <c r="D31" s="94"/>
+      <c r="E31" s="97"/>
+      <c r="F31" s="90"/>
+      <c r="G31" s="90"/>
+      <c r="H31" s="90"/>
+      <c r="I31" s="90"/>
+      <c r="J31" s="90"/>
+      <c r="K31" s="90"/>
+      <c r="L31" s="90"/>
+      <c r="M31" s="90"/>
+      <c r="N31" s="90"/>
+      <c r="O31" s="90"/>
+      <c r="P31" s="90"/>
+      <c r="Q31" s="90"/>
+      <c r="R31" s="90"/>
+      <c r="S31" s="90"/>
+      <c r="T31" s="90"/>
+      <c r="U31" s="90"/>
+      <c r="V31" s="90"/>
+      <c r="W31" s="90"/>
+      <c r="X31" s="65"/>
+      <c r="Y31" s="65"/>
+      <c r="Z31" s="65"/>
+      <c r="AA31" s="65"/>
+      <c r="AB31" s="65"/>
+      <c r="AC31" s="65"/>
     </row>
     <row r="32" spans="1:29">
-      <c r="A32" s="80">
+      <c r="A32" s="73">
         <v>19</v>
       </c>
-      <c r="B32" s="105" t="s">
+      <c r="B32" s="98" t="s">
         <v>155</v>
       </c>
-      <c r="C32" s="106">
+      <c r="C32" s="99">
         <v>7</v>
       </c>
-      <c r="D32" s="101"/>
-      <c r="E32" s="104"/>
-      <c r="F32" s="97"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="97"/>
-      <c r="I32" s="97"/>
-      <c r="J32" s="97"/>
-      <c r="K32" s="97"/>
-      <c r="L32" s="97"/>
-      <c r="M32" s="97"/>
-      <c r="N32" s="97"/>
-      <c r="O32" s="97"/>
-      <c r="P32" s="97"/>
-      <c r="Q32" s="97"/>
-      <c r="R32" s="97"/>
-      <c r="S32" s="97"/>
-      <c r="T32" s="97"/>
-      <c r="U32" s="97"/>
-      <c r="V32" s="97"/>
-      <c r="W32" s="97"/>
-      <c r="X32" s="71"/>
-      <c r="Y32" s="71"/>
-      <c r="Z32" s="71"/>
-      <c r="AA32" s="71"/>
-      <c r="AB32" s="71"/>
-      <c r="AC32" s="71"/>
+      <c r="D32" s="94"/>
+      <c r="E32" s="97"/>
+      <c r="F32" s="90"/>
+      <c r="G32" s="90"/>
+      <c r="H32" s="90"/>
+      <c r="I32" s="90"/>
+      <c r="J32" s="90"/>
+      <c r="K32" s="90"/>
+      <c r="L32" s="90"/>
+      <c r="M32" s="90"/>
+      <c r="N32" s="90"/>
+      <c r="O32" s="90"/>
+      <c r="P32" s="90"/>
+      <c r="Q32" s="90"/>
+      <c r="R32" s="90"/>
+      <c r="S32" s="90"/>
+      <c r="T32" s="90"/>
+      <c r="U32" s="90"/>
+      <c r="V32" s="90"/>
+      <c r="W32" s="90"/>
+      <c r="X32" s="65"/>
+      <c r="Y32" s="65"/>
+      <c r="Z32" s="65"/>
+      <c r="AA32" s="65"/>
+      <c r="AB32" s="65"/>
+      <c r="AC32" s="65"/>
     </row>
     <row r="33" spans="1:29">
-      <c r="A33" s="80">
+      <c r="A33" s="73">
         <v>20</v>
       </c>
-      <c r="B33" s="113" t="s">
+      <c r="B33" s="106" t="s">
         <v>156</v>
       </c>
-      <c r="C33" s="114">
+      <c r="C33" s="107">
         <v>5</v>
       </c>
-      <c r="D33" s="101"/>
-      <c r="E33" s="104"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="97"/>
-      <c r="J33" s="97"/>
-      <c r="K33" s="97"/>
-      <c r="L33" s="97"/>
-      <c r="M33" s="97"/>
-      <c r="N33" s="97"/>
-      <c r="O33" s="97"/>
-      <c r="P33" s="97"/>
-      <c r="Q33" s="97"/>
-      <c r="R33" s="97"/>
-      <c r="S33" s="97"/>
-      <c r="T33" s="97"/>
-      <c r="U33" s="97"/>
-      <c r="V33" s="97"/>
-      <c r="W33" s="97"/>
-      <c r="X33" s="71"/>
-      <c r="Y33" s="71"/>
-      <c r="Z33" s="71"/>
-      <c r="AA33" s="71"/>
-      <c r="AB33" s="71"/>
-      <c r="AC33" s="71"/>
+      <c r="D33" s="94"/>
+      <c r="E33" s="97"/>
+      <c r="F33" s="90"/>
+      <c r="G33" s="90"/>
+      <c r="H33" s="90"/>
+      <c r="I33" s="90"/>
+      <c r="J33" s="90"/>
+      <c r="K33" s="90"/>
+      <c r="L33" s="90"/>
+      <c r="M33" s="90"/>
+      <c r="N33" s="90"/>
+      <c r="O33" s="90"/>
+      <c r="P33" s="90"/>
+      <c r="Q33" s="90"/>
+      <c r="R33" s="90"/>
+      <c r="S33" s="90"/>
+      <c r="T33" s="90"/>
+      <c r="U33" s="90"/>
+      <c r="V33" s="90"/>
+      <c r="W33" s="90"/>
+      <c r="X33" s="65"/>
+      <c r="Y33" s="65"/>
+      <c r="Z33" s="65"/>
+      <c r="AA33" s="65"/>
+      <c r="AB33" s="65"/>
+      <c r="AC33" s="65"/>
     </row>
     <row r="34" spans="1:29">
-      <c r="A34" s="80">
+      <c r="A34" s="73">
         <v>21</v>
       </c>
-      <c r="B34" s="115" t="s">
+      <c r="B34" s="108" t="s">
         <v>157</v>
       </c>
-      <c r="C34" s="114">
+      <c r="C34" s="107">
         <v>5</v>
       </c>
-      <c r="D34" s="101"/>
-      <c r="E34" s="104"/>
-      <c r="F34" s="97"/>
-      <c r="G34" s="97"/>
-      <c r="H34" s="97"/>
-      <c r="I34" s="97"/>
-      <c r="J34" s="97"/>
-      <c r="K34" s="97"/>
-      <c r="L34" s="97"/>
-      <c r="M34" s="97"/>
-      <c r="N34" s="97"/>
-      <c r="O34" s="97"/>
-      <c r="P34" s="97"/>
-      <c r="Q34" s="97"/>
-      <c r="R34" s="97"/>
-      <c r="S34" s="97"/>
-      <c r="T34" s="97"/>
-      <c r="U34" s="97"/>
-      <c r="V34" s="97"/>
-      <c r="W34" s="97"/>
-      <c r="X34" s="71"/>
-      <c r="Y34" s="71"/>
-      <c r="Z34" s="71"/>
-      <c r="AA34" s="71"/>
-      <c r="AB34" s="71"/>
-      <c r="AC34" s="71"/>
+      <c r="D34" s="94"/>
+      <c r="E34" s="97"/>
+      <c r="F34" s="90"/>
+      <c r="G34" s="90"/>
+      <c r="H34" s="90"/>
+      <c r="I34" s="90"/>
+      <c r="J34" s="90"/>
+      <c r="K34" s="90"/>
+      <c r="L34" s="90"/>
+      <c r="M34" s="90"/>
+      <c r="N34" s="90"/>
+      <c r="O34" s="90"/>
+      <c r="P34" s="90"/>
+      <c r="Q34" s="90"/>
+      <c r="R34" s="90"/>
+      <c r="S34" s="90"/>
+      <c r="T34" s="90"/>
+      <c r="U34" s="90"/>
+      <c r="V34" s="90"/>
+      <c r="W34" s="90"/>
+      <c r="X34" s="65"/>
+      <c r="Y34" s="65"/>
+      <c r="Z34" s="65"/>
+      <c r="AA34" s="65"/>
+      <c r="AB34" s="65"/>
+      <c r="AC34" s="65"/>
     </row>
     <row r="35" spans="1:29">
-      <c r="A35" s="80">
+      <c r="A35" s="73">
         <v>23</v>
       </c>
-      <c r="B35" s="116" t="s">
+      <c r="B35" s="109" t="s">
         <v>159</v>
       </c>
-      <c r="C35" s="106">
+      <c r="C35" s="99">
         <v>3</v>
       </c>
-      <c r="D35" s="101"/>
-      <c r="E35" s="104"/>
-      <c r="F35" s="97"/>
-      <c r="G35" s="97"/>
-      <c r="H35" s="97"/>
-      <c r="I35" s="97"/>
-      <c r="J35" s="97"/>
-      <c r="K35" s="97"/>
-      <c r="L35" s="97"/>
-      <c r="M35" s="97"/>
-      <c r="N35" s="97"/>
-      <c r="O35" s="97"/>
-      <c r="P35" s="97"/>
-      <c r="Q35" s="97"/>
-      <c r="R35" s="97"/>
-      <c r="S35" s="97"/>
-      <c r="T35" s="97"/>
-      <c r="U35" s="97"/>
-      <c r="V35" s="97"/>
-      <c r="W35" s="97"/>
-      <c r="X35" s="71"/>
-      <c r="Y35" s="71"/>
-      <c r="Z35" s="71"/>
-      <c r="AA35" s="71"/>
-      <c r="AB35" s="71"/>
-      <c r="AC35" s="71"/>
+      <c r="D35" s="94"/>
+      <c r="E35" s="97"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="90"/>
+      <c r="H35" s="90"/>
+      <c r="I35" s="90"/>
+      <c r="J35" s="90"/>
+      <c r="K35" s="90"/>
+      <c r="L35" s="90"/>
+      <c r="M35" s="90"/>
+      <c r="N35" s="90"/>
+      <c r="O35" s="90"/>
+      <c r="P35" s="90"/>
+      <c r="Q35" s="90"/>
+      <c r="R35" s="90"/>
+      <c r="S35" s="90"/>
+      <c r="T35" s="90"/>
+      <c r="U35" s="90"/>
+      <c r="V35" s="90"/>
+      <c r="W35" s="90"/>
+      <c r="X35" s="65"/>
+      <c r="Y35" s="65"/>
+      <c r="Z35" s="65"/>
+      <c r="AA35" s="65"/>
+      <c r="AB35" s="65"/>
+      <c r="AC35" s="65"/>
     </row>
     <row r="36" spans="1:29">
-      <c r="A36" s="80">
+      <c r="A36" s="73">
         <v>24</v>
       </c>
-      <c r="B36" s="117" t="s">
+      <c r="B36" s="110" t="s">
         <v>160</v>
       </c>
-      <c r="C36" s="118">
+      <c r="C36" s="111">
         <v>10</v>
       </c>
-      <c r="D36" s="101"/>
-      <c r="E36" s="119"/>
-      <c r="F36" s="120"/>
-      <c r="G36" s="120"/>
-      <c r="H36" s="120"/>
-      <c r="I36" s="120"/>
-      <c r="J36" s="120"/>
-      <c r="K36" s="120"/>
-      <c r="L36" s="120"/>
-      <c r="M36" s="120"/>
-      <c r="N36" s="120"/>
-      <c r="O36" s="120"/>
-      <c r="P36" s="120"/>
-      <c r="Q36" s="120"/>
-      <c r="R36" s="120"/>
-      <c r="S36" s="120"/>
-      <c r="T36" s="97"/>
-      <c r="U36" s="97"/>
-      <c r="V36" s="97"/>
-      <c r="W36" s="97"/>
-      <c r="X36" s="71"/>
-      <c r="Y36" s="71"/>
-      <c r="Z36" s="71"/>
-      <c r="AA36" s="71"/>
-      <c r="AB36" s="71"/>
-      <c r="AC36" s="71"/>
+      <c r="D36" s="94"/>
+      <c r="E36" s="112"/>
+      <c r="F36" s="113"/>
+      <c r="G36" s="113"/>
+      <c r="H36" s="113"/>
+      <c r="I36" s="113"/>
+      <c r="J36" s="113"/>
+      <c r="K36" s="113"/>
+      <c r="L36" s="113"/>
+      <c r="M36" s="113"/>
+      <c r="N36" s="113"/>
+      <c r="O36" s="113"/>
+      <c r="P36" s="113"/>
+      <c r="Q36" s="113"/>
+      <c r="R36" s="113"/>
+      <c r="S36" s="113"/>
+      <c r="T36" s="90"/>
+      <c r="U36" s="90"/>
+      <c r="V36" s="90"/>
+      <c r="W36" s="90"/>
+      <c r="X36" s="65"/>
+      <c r="Y36" s="65"/>
+      <c r="Z36" s="65"/>
+      <c r="AA36" s="65"/>
+      <c r="AB36" s="65"/>
+      <c r="AC36" s="65"/>
     </row>
     <row r="37" spans="1:29">
-      <c r="A37" s="80">
+      <c r="A37" s="73">
         <v>25</v>
       </c>
-      <c r="B37" s="121" t="s">
+      <c r="B37" s="114" t="s">
         <v>161</v>
       </c>
-      <c r="C37" s="118">
+      <c r="C37" s="111">
         <v>5</v>
       </c>
-      <c r="D37" s="101"/>
-      <c r="E37" s="119"/>
-      <c r="F37" s="120"/>
-      <c r="G37" s="120"/>
-      <c r="H37" s="120"/>
-      <c r="I37" s="120"/>
-      <c r="J37" s="120"/>
-      <c r="K37" s="120"/>
-      <c r="L37" s="120"/>
-      <c r="M37" s="120"/>
-      <c r="N37" s="120"/>
-      <c r="O37" s="120"/>
-      <c r="P37" s="120"/>
-      <c r="Q37" s="120"/>
-      <c r="R37" s="120"/>
-      <c r="S37" s="120"/>
-      <c r="T37" s="97"/>
-      <c r="U37" s="97"/>
-      <c r="V37" s="97"/>
-      <c r="W37" s="97"/>
-      <c r="X37" s="71"/>
-      <c r="Y37" s="71"/>
-      <c r="Z37" s="71"/>
-      <c r="AA37" s="71"/>
-      <c r="AB37" s="71"/>
-      <c r="AC37" s="71"/>
+      <c r="D37" s="94"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="113"/>
+      <c r="G37" s="113"/>
+      <c r="H37" s="113"/>
+      <c r="I37" s="113"/>
+      <c r="J37" s="113"/>
+      <c r="K37" s="113"/>
+      <c r="L37" s="113"/>
+      <c r="M37" s="113"/>
+      <c r="N37" s="113"/>
+      <c r="O37" s="113"/>
+      <c r="P37" s="113"/>
+      <c r="Q37" s="113"/>
+      <c r="R37" s="113"/>
+      <c r="S37" s="113"/>
+      <c r="T37" s="90"/>
+      <c r="U37" s="90"/>
+      <c r="V37" s="90"/>
+      <c r="W37" s="90"/>
+      <c r="X37" s="65"/>
+      <c r="Y37" s="65"/>
+      <c r="Z37" s="65"/>
+      <c r="AA37" s="65"/>
+      <c r="AB37" s="65"/>
+      <c r="AC37" s="65"/>
     </row>
     <row r="38" spans="1:29">
-      <c r="A38" s="80">
+      <c r="A38" s="73">
         <v>26</v>
       </c>
-      <c r="B38" s="122" t="s">
+      <c r="B38" s="115" t="s">
         <v>162</v>
       </c>
-      <c r="C38" s="114">
+      <c r="C38" s="107">
         <v>6</v>
       </c>
-      <c r="D38" s="101"/>
-      <c r="E38" s="119"/>
-      <c r="F38" s="120"/>
-      <c r="G38" s="120"/>
-      <c r="H38" s="120"/>
-      <c r="I38" s="120"/>
-      <c r="J38" s="120"/>
-      <c r="K38" s="120"/>
-      <c r="L38" s="120"/>
-      <c r="M38" s="120"/>
-      <c r="N38" s="120"/>
-      <c r="O38" s="120"/>
-      <c r="P38" s="120"/>
-      <c r="Q38" s="120"/>
-      <c r="R38" s="120"/>
-      <c r="S38" s="120"/>
-      <c r="T38" s="97"/>
-      <c r="U38" s="97"/>
-      <c r="V38" s="97"/>
-      <c r="W38" s="97"/>
-      <c r="X38" s="71"/>
-      <c r="Y38" s="71"/>
-      <c r="Z38" s="71"/>
-      <c r="AA38" s="71"/>
-      <c r="AB38" s="71"/>
-      <c r="AC38" s="71"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="113"/>
+      <c r="G38" s="113"/>
+      <c r="H38" s="113"/>
+      <c r="I38" s="113"/>
+      <c r="J38" s="113"/>
+      <c r="K38" s="113"/>
+      <c r="L38" s="113"/>
+      <c r="M38" s="113"/>
+      <c r="N38" s="113"/>
+      <c r="O38" s="113"/>
+      <c r="P38" s="113"/>
+      <c r="Q38" s="113"/>
+      <c r="R38" s="113"/>
+      <c r="S38" s="113"/>
+      <c r="T38" s="90"/>
+      <c r="U38" s="90"/>
+      <c r="V38" s="90"/>
+      <c r="W38" s="90"/>
+      <c r="X38" s="65"/>
+      <c r="Y38" s="65"/>
+      <c r="Z38" s="65"/>
+      <c r="AA38" s="65"/>
+      <c r="AB38" s="65"/>
+      <c r="AC38" s="65"/>
     </row>
     <row r="39" spans="1:29">
-      <c r="A39" s="80">
+      <c r="A39" s="73">
         <v>27</v>
       </c>
-      <c r="B39" s="121" t="s">
+      <c r="B39" s="114" t="s">
         <v>163</v>
       </c>
-      <c r="C39" s="118">
+      <c r="C39" s="111">
         <v>5</v>
       </c>
-      <c r="D39" s="101"/>
-      <c r="E39" s="119"/>
-      <c r="F39" s="120"/>
-      <c r="G39" s="120"/>
-      <c r="H39" s="120"/>
-      <c r="I39" s="120"/>
-      <c r="J39" s="120"/>
-      <c r="K39" s="120"/>
-      <c r="L39" s="120"/>
-      <c r="M39" s="120"/>
-      <c r="N39" s="120"/>
-      <c r="O39" s="120"/>
-      <c r="P39" s="120"/>
-      <c r="Q39" s="120"/>
-      <c r="R39" s="120"/>
-      <c r="S39" s="120"/>
-      <c r="T39" s="97"/>
-      <c r="U39" s="97"/>
-      <c r="V39" s="97"/>
-      <c r="W39" s="97"/>
-      <c r="X39" s="71"/>
-      <c r="Y39" s="71"/>
-      <c r="Z39" s="71"/>
-      <c r="AA39" s="71"/>
-      <c r="AB39" s="71"/>
-      <c r="AC39" s="71"/>
+      <c r="D39" s="94"/>
+      <c r="E39" s="112"/>
+      <c r="F39" s="113"/>
+      <c r="G39" s="113"/>
+      <c r="H39" s="113"/>
+      <c r="I39" s="113"/>
+      <c r="J39" s="113"/>
+      <c r="K39" s="113"/>
+      <c r="L39" s="113"/>
+      <c r="M39" s="113"/>
+      <c r="N39" s="113"/>
+      <c r="O39" s="113"/>
+      <c r="P39" s="113"/>
+      <c r="Q39" s="113"/>
+      <c r="R39" s="113"/>
+      <c r="S39" s="113"/>
+      <c r="T39" s="90"/>
+      <c r="U39" s="90"/>
+      <c r="V39" s="90"/>
+      <c r="W39" s="90"/>
+      <c r="X39" s="65"/>
+      <c r="Y39" s="65"/>
+      <c r="Z39" s="65"/>
+      <c r="AA39" s="65"/>
+      <c r="AB39" s="65"/>
+      <c r="AC39" s="65"/>
     </row>
     <row r="40" spans="1:29">
-      <c r="A40" s="80">
+      <c r="A40" s="73">
         <v>28</v>
       </c>
-      <c r="B40" s="123" t="s">
+      <c r="B40" s="116" t="s">
         <v>174</v>
       </c>
-      <c r="C40" s="118">
+      <c r="C40" s="111">
         <v>5</v>
       </c>
-      <c r="D40" s="101"/>
-      <c r="E40" s="119"/>
-      <c r="F40" s="120"/>
-      <c r="G40" s="120"/>
-      <c r="H40" s="120"/>
-      <c r="I40" s="120"/>
-      <c r="J40" s="120"/>
-      <c r="K40" s="120"/>
-      <c r="L40" s="120"/>
-      <c r="M40" s="120"/>
-      <c r="N40" s="120"/>
-      <c r="O40" s="120"/>
-      <c r="P40" s="120"/>
-      <c r="Q40" s="120"/>
-      <c r="R40" s="120"/>
-      <c r="S40" s="120"/>
-      <c r="T40" s="97"/>
-      <c r="U40" s="97"/>
-      <c r="V40" s="97"/>
-      <c r="W40" s="97"/>
-      <c r="X40" s="71"/>
-      <c r="Y40" s="71"/>
-      <c r="Z40" s="71"/>
-      <c r="AA40" s="71"/>
-      <c r="AB40" s="71"/>
-      <c r="AC40" s="71"/>
+      <c r="D40" s="94"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="113"/>
+      <c r="G40" s="113"/>
+      <c r="H40" s="113"/>
+      <c r="I40" s="113"/>
+      <c r="J40" s="113"/>
+      <c r="K40" s="113"/>
+      <c r="L40" s="113"/>
+      <c r="M40" s="113"/>
+      <c r="N40" s="113"/>
+      <c r="O40" s="113"/>
+      <c r="P40" s="113"/>
+      <c r="Q40" s="113"/>
+      <c r="R40" s="113"/>
+      <c r="S40" s="113"/>
+      <c r="T40" s="90"/>
+      <c r="U40" s="90"/>
+      <c r="V40" s="90"/>
+      <c r="W40" s="90"/>
+      <c r="X40" s="65"/>
+      <c r="Y40" s="65"/>
+      <c r="Z40" s="65"/>
+      <c r="AA40" s="65"/>
+      <c r="AB40" s="65"/>
+      <c r="AC40" s="65"/>
     </row>
     <row r="41" spans="1:29">
-      <c r="A41" s="80">
+      <c r="A41" s="73">
         <v>29</v>
       </c>
-      <c r="B41" s="123" t="s">
+      <c r="B41" s="116" t="s">
         <v>176</v>
       </c>
-      <c r="C41" s="118">
+      <c r="C41" s="111">
         <v>3</v>
       </c>
-      <c r="D41" s="101"/>
-      <c r="E41" s="119"/>
-      <c r="F41" s="120"/>
-      <c r="G41" s="120"/>
-      <c r="H41" s="120"/>
-      <c r="I41" s="120"/>
-      <c r="J41" s="120"/>
-      <c r="K41" s="120"/>
-      <c r="L41" s="120"/>
-      <c r="M41" s="120"/>
-      <c r="N41" s="120"/>
-      <c r="O41" s="120"/>
-      <c r="P41" s="120"/>
-      <c r="Q41" s="120"/>
-      <c r="R41" s="120"/>
-      <c r="S41" s="120"/>
-      <c r="T41" s="97"/>
-      <c r="U41" s="97"/>
-      <c r="V41" s="97"/>
-      <c r="W41" s="97"/>
-      <c r="X41" s="71"/>
-      <c r="Y41" s="71"/>
-      <c r="Z41" s="71"/>
-      <c r="AA41" s="71"/>
-      <c r="AB41" s="71"/>
-      <c r="AC41" s="71"/>
+      <c r="D41" s="94"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="113"/>
+      <c r="G41" s="113"/>
+      <c r="H41" s="113"/>
+      <c r="I41" s="113"/>
+      <c r="J41" s="113"/>
+      <c r="K41" s="113"/>
+      <c r="L41" s="113"/>
+      <c r="M41" s="113"/>
+      <c r="N41" s="113"/>
+      <c r="O41" s="113"/>
+      <c r="P41" s="113"/>
+      <c r="Q41" s="113"/>
+      <c r="R41" s="113"/>
+      <c r="S41" s="113"/>
+      <c r="T41" s="90"/>
+      <c r="U41" s="90"/>
+      <c r="V41" s="90"/>
+      <c r="W41" s="90"/>
+      <c r="X41" s="65"/>
+      <c r="Y41" s="65"/>
+      <c r="Z41" s="65"/>
+      <c r="AA41" s="65"/>
+      <c r="AB41" s="65"/>
+      <c r="AC41" s="65"/>
     </row>
     <row r="42" spans="1:29">
-      <c r="A42" s="80">
+      <c r="A42" s="73">
         <v>29</v>
       </c>
-      <c r="B42" s="123" t="s">
+      <c r="B42" s="116" t="s">
         <v>164</v>
       </c>
-      <c r="C42" s="118">
+      <c r="C42" s="111">
         <v>6</v>
       </c>
-      <c r="D42" s="101"/>
-      <c r="E42" s="119"/>
-      <c r="F42" s="120"/>
-      <c r="G42" s="120"/>
-      <c r="H42" s="120"/>
-      <c r="I42" s="120"/>
-      <c r="J42" s="120"/>
-      <c r="K42" s="120"/>
-      <c r="L42" s="120"/>
-      <c r="M42" s="120"/>
-      <c r="N42" s="120"/>
-      <c r="O42" s="120"/>
-      <c r="P42" s="120"/>
-      <c r="Q42" s="120"/>
-      <c r="R42" s="120"/>
-      <c r="S42" s="120"/>
-      <c r="T42" s="97"/>
-      <c r="U42" s="97"/>
-      <c r="V42" s="97"/>
-      <c r="W42" s="97"/>
-      <c r="X42" s="71"/>
-      <c r="Y42" s="71"/>
-      <c r="Z42" s="71"/>
-      <c r="AA42" s="71"/>
-      <c r="AB42" s="71"/>
-      <c r="AC42" s="71"/>
+      <c r="D42" s="94"/>
+      <c r="E42" s="112"/>
+      <c r="F42" s="113"/>
+      <c r="G42" s="113"/>
+      <c r="H42" s="113"/>
+      <c r="I42" s="113"/>
+      <c r="J42" s="113"/>
+      <c r="K42" s="113"/>
+      <c r="L42" s="113"/>
+      <c r="M42" s="113"/>
+      <c r="N42" s="113"/>
+      <c r="O42" s="113"/>
+      <c r="P42" s="113"/>
+      <c r="Q42" s="113"/>
+      <c r="R42" s="113"/>
+      <c r="S42" s="113"/>
+      <c r="T42" s="90"/>
+      <c r="U42" s="90"/>
+      <c r="V42" s="90"/>
+      <c r="W42" s="90"/>
+      <c r="X42" s="65"/>
+      <c r="Y42" s="65"/>
+      <c r="Z42" s="65"/>
+      <c r="AA42" s="65"/>
+      <c r="AB42" s="65"/>
+      <c r="AC42" s="65"/>
     </row>
     <row r="43" spans="1:29">
-      <c r="A43" s="80">
+      <c r="A43" s="73">
         <v>30</v>
       </c>
-      <c r="B43" s="123" t="s">
+      <c r="B43" s="116" t="s">
         <v>165</v>
       </c>
-      <c r="C43" s="118">
+      <c r="C43" s="111">
         <v>8</v>
       </c>
-      <c r="D43" s="101"/>
-      <c r="E43" s="119"/>
-      <c r="F43" s="120"/>
-      <c r="G43" s="120"/>
-      <c r="H43" s="120"/>
-      <c r="I43" s="120"/>
-      <c r="J43" s="120"/>
-      <c r="K43" s="120"/>
-      <c r="L43" s="120"/>
-      <c r="M43" s="120"/>
-      <c r="N43" s="120"/>
-      <c r="O43" s="120"/>
-      <c r="P43" s="120"/>
-      <c r="Q43" s="120"/>
-      <c r="R43" s="120"/>
-      <c r="S43" s="120"/>
-      <c r="T43" s="97"/>
-      <c r="U43" s="97"/>
-      <c r="V43" s="97"/>
-      <c r="W43" s="97"/>
-      <c r="X43" s="71"/>
-      <c r="Y43" s="71"/>
-      <c r="Z43" s="71"/>
-      <c r="AA43" s="71"/>
-      <c r="AB43" s="71"/>
-      <c r="AC43" s="71"/>
+      <c r="D43" s="94"/>
+      <c r="E43" s="112"/>
+      <c r="F43" s="113"/>
+      <c r="G43" s="113"/>
+      <c r="H43" s="113"/>
+      <c r="I43" s="113"/>
+      <c r="J43" s="113"/>
+      <c r="K43" s="113"/>
+      <c r="L43" s="113"/>
+      <c r="M43" s="113"/>
+      <c r="N43" s="113"/>
+      <c r="O43" s="113"/>
+      <c r="P43" s="113"/>
+      <c r="Q43" s="113"/>
+      <c r="R43" s="113"/>
+      <c r="S43" s="113"/>
+      <c r="T43" s="90"/>
+      <c r="U43" s="90"/>
+      <c r="V43" s="90"/>
+      <c r="W43" s="90"/>
+      <c r="X43" s="65"/>
+      <c r="Y43" s="65"/>
+      <c r="Z43" s="65"/>
+      <c r="AA43" s="65"/>
+      <c r="AB43" s="65"/>
+      <c r="AC43" s="65"/>
     </row>
     <row r="44" spans="1:29">
-      <c r="A44" s="80">
+      <c r="A44" s="73">
         <v>31</v>
       </c>
-      <c r="B44" s="115" t="s">
+      <c r="B44" s="108" t="s">
         <v>166</v>
       </c>
-      <c r="C44" s="124">
+      <c r="C44" s="117">
         <v>4</v>
       </c>
-      <c r="D44" s="101"/>
-      <c r="E44" s="119"/>
-      <c r="F44" s="101"/>
-      <c r="G44" s="101"/>
-      <c r="H44" s="101"/>
-      <c r="I44" s="101"/>
-      <c r="J44" s="101"/>
-      <c r="K44" s="101"/>
-      <c r="L44" s="120"/>
-      <c r="M44" s="101"/>
-      <c r="N44" s="101"/>
-      <c r="O44" s="101"/>
-      <c r="P44" s="101"/>
-      <c r="Q44" s="101"/>
-      <c r="R44" s="101"/>
-      <c r="S44" s="101"/>
-      <c r="T44" s="97"/>
-      <c r="U44" s="97"/>
-      <c r="V44" s="97"/>
-      <c r="W44" s="97"/>
-      <c r="X44" s="71"/>
-      <c r="Y44" s="71"/>
-      <c r="Z44" s="71"/>
-      <c r="AA44" s="71"/>
-      <c r="AB44" s="71"/>
-      <c r="AC44" s="71"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="112"/>
+      <c r="F44" s="94"/>
+      <c r="G44" s="94"/>
+      <c r="H44" s="94"/>
+      <c r="I44" s="94"/>
+      <c r="J44" s="94"/>
+      <c r="K44" s="94"/>
+      <c r="L44" s="113"/>
+      <c r="M44" s="94"/>
+      <c r="N44" s="94"/>
+      <c r="O44" s="94"/>
+      <c r="P44" s="94"/>
+      <c r="Q44" s="94"/>
+      <c r="R44" s="94"/>
+      <c r="S44" s="94"/>
+      <c r="T44" s="90"/>
+      <c r="U44" s="90"/>
+      <c r="V44" s="90"/>
+      <c r="W44" s="90"/>
+      <c r="X44" s="65"/>
+      <c r="Y44" s="65"/>
+      <c r="Z44" s="65"/>
+      <c r="AA44" s="65"/>
+      <c r="AB44" s="65"/>
+      <c r="AC44" s="65"/>
     </row>
     <row r="45" spans="1:29">
-      <c r="A45" s="80">
+      <c r="A45" s="73">
         <v>32</v>
       </c>
-      <c r="B45" s="125" t="s">
+      <c r="B45" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="C45" s="114">
+      <c r="C45" s="107">
         <v>4</v>
       </c>
-      <c r="D45" s="101"/>
-      <c r="E45" s="119"/>
-      <c r="F45" s="101"/>
-      <c r="G45" s="101"/>
-      <c r="H45" s="101"/>
-      <c r="I45" s="101"/>
-      <c r="J45" s="101"/>
-      <c r="K45" s="101"/>
-      <c r="L45" s="120"/>
-      <c r="M45" s="101"/>
-      <c r="N45" s="101"/>
-      <c r="O45" s="101"/>
-      <c r="P45" s="101"/>
-      <c r="Q45" s="101"/>
-      <c r="R45" s="101"/>
-      <c r="S45" s="101"/>
-      <c r="T45" s="97"/>
-      <c r="U45" s="97"/>
-      <c r="V45" s="97"/>
-      <c r="W45" s="97"/>
-      <c r="X45" s="71"/>
-      <c r="Y45" s="71"/>
-      <c r="Z45" s="71"/>
-      <c r="AA45" s="71"/>
-      <c r="AB45" s="71"/>
-      <c r="AC45" s="71"/>
+      <c r="D45" s="94"/>
+      <c r="E45" s="112"/>
+      <c r="F45" s="94"/>
+      <c r="G45" s="94"/>
+      <c r="H45" s="94"/>
+      <c r="I45" s="94"/>
+      <c r="J45" s="94"/>
+      <c r="K45" s="94"/>
+      <c r="L45" s="113"/>
+      <c r="M45" s="94"/>
+      <c r="N45" s="94"/>
+      <c r="O45" s="94"/>
+      <c r="P45" s="94"/>
+      <c r="Q45" s="94"/>
+      <c r="R45" s="94"/>
+      <c r="S45" s="94"/>
+      <c r="T45" s="90"/>
+      <c r="U45" s="90"/>
+      <c r="V45" s="90"/>
+      <c r="W45" s="90"/>
+      <c r="X45" s="65"/>
+      <c r="Y45" s="65"/>
+      <c r="Z45" s="65"/>
+      <c r="AA45" s="65"/>
+      <c r="AB45" s="65"/>
+      <c r="AC45" s="65"/>
     </row>
     <row r="46" spans="1:29">
-      <c r="A46" s="80">
+      <c r="A46" s="73">
         <v>33</v>
       </c>
-      <c r="B46" s="117" t="s">
+      <c r="B46" s="110" t="s">
         <v>168</v>
       </c>
-      <c r="C46" s="118">
+      <c r="C46" s="111">
         <v>4</v>
       </c>
-      <c r="D46" s="101"/>
-      <c r="E46" s="119"/>
-      <c r="F46" s="101"/>
-      <c r="G46" s="101"/>
-      <c r="H46" s="101"/>
-      <c r="I46" s="101"/>
-      <c r="J46" s="101"/>
-      <c r="K46" s="101"/>
-      <c r="L46" s="120"/>
-      <c r="M46" s="101"/>
-      <c r="N46" s="101"/>
-      <c r="O46" s="101"/>
-      <c r="P46" s="101"/>
-      <c r="Q46" s="101"/>
-      <c r="R46" s="101"/>
-      <c r="S46" s="101"/>
-      <c r="T46" s="97"/>
-      <c r="U46" s="97"/>
-      <c r="V46" s="97"/>
-      <c r="W46" s="97"/>
-      <c r="X46" s="71"/>
-      <c r="Y46" s="71"/>
-      <c r="Z46" s="71"/>
-      <c r="AA46" s="71"/>
-      <c r="AB46" s="71"/>
-      <c r="AC46" s="71"/>
+      <c r="D46" s="94"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="94"/>
+      <c r="G46" s="94"/>
+      <c r="H46" s="94"/>
+      <c r="I46" s="94"/>
+      <c r="J46" s="94"/>
+      <c r="K46" s="94"/>
+      <c r="L46" s="113"/>
+      <c r="M46" s="94"/>
+      <c r="N46" s="94"/>
+      <c r="O46" s="94"/>
+      <c r="P46" s="94"/>
+      <c r="Q46" s="94"/>
+      <c r="R46" s="94"/>
+      <c r="S46" s="94"/>
+      <c r="T46" s="90"/>
+      <c r="U46" s="90"/>
+      <c r="V46" s="90"/>
+      <c r="W46" s="90"/>
+      <c r="X46" s="65"/>
+      <c r="Y46" s="65"/>
+      <c r="Z46" s="65"/>
+      <c r="AA46" s="65"/>
+      <c r="AB46" s="65"/>
+      <c r="AC46" s="65"/>
     </row>
     <row r="47" spans="1:29" ht="15" thickBot="1">
-      <c r="A47" s="80">
+      <c r="A47" s="73">
         <v>34</v>
       </c>
-      <c r="B47" s="117" t="s">
+      <c r="B47" s="110" t="s">
         <v>169</v>
       </c>
-      <c r="C47" s="114">
+      <c r="C47" s="107">
         <v>12</v>
       </c>
-      <c r="D47" s="101"/>
-      <c r="E47" s="119"/>
-      <c r="F47" s="70"/>
-      <c r="G47" s="70"/>
-      <c r="H47" s="70"/>
-      <c r="I47" s="70"/>
-      <c r="J47" s="70"/>
-      <c r="K47" s="70"/>
-      <c r="L47" s="120"/>
-      <c r="M47" s="70"/>
-      <c r="N47" s="70"/>
-      <c r="O47" s="70"/>
-      <c r="P47" s="70"/>
-      <c r="Q47" s="70"/>
-      <c r="R47" s="70"/>
-      <c r="S47" s="70"/>
-      <c r="T47" s="103"/>
-      <c r="U47" s="126"/>
-      <c r="V47" s="126"/>
-      <c r="W47" s="126"/>
-      <c r="X47" s="71"/>
-      <c r="Y47" s="71"/>
-      <c r="Z47" s="71"/>
-      <c r="AA47" s="71"/>
-      <c r="AB47" s="71"/>
-      <c r="AC47" s="71"/>
+      <c r="D47" s="94"/>
+      <c r="E47" s="112"/>
+      <c r="F47" s="64"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="64"/>
+      <c r="J47" s="64"/>
+      <c r="K47" s="64"/>
+      <c r="L47" s="113"/>
+      <c r="M47" s="64"/>
+      <c r="N47" s="64"/>
+      <c r="O47" s="64"/>
+      <c r="P47" s="64"/>
+      <c r="Q47" s="64"/>
+      <c r="R47" s="64"/>
+      <c r="S47" s="64"/>
+      <c r="T47" s="96"/>
+      <c r="U47" s="119"/>
+      <c r="V47" s="119"/>
+      <c r="W47" s="119"/>
+      <c r="X47" s="65"/>
+      <c r="Y47" s="65"/>
+      <c r="Z47" s="65"/>
+      <c r="AA47" s="65"/>
+      <c r="AB47" s="65"/>
+      <c r="AC47" s="65"/>
     </row>
     <row r="48" spans="1:29" ht="54" thickTop="1">
-      <c r="A48" s="127"/>
-      <c r="B48" s="128" t="s">
+      <c r="A48" s="120"/>
+      <c r="B48" s="121" t="s">
         <v>77</v>
       </c>
-      <c r="C48" s="129"/>
-      <c r="D48" s="129"/>
-      <c r="E48" s="130"/>
-      <c r="F48" s="129"/>
-      <c r="G48" s="129"/>
-      <c r="H48" s="129"/>
-      <c r="I48" s="129"/>
-      <c r="J48" s="129"/>
-      <c r="K48" s="129"/>
-      <c r="L48" s="131"/>
-      <c r="M48" s="129"/>
-      <c r="N48" s="129"/>
-      <c r="O48" s="129"/>
-      <c r="P48" s="132" t="s">
+      <c r="C48" s="122"/>
+      <c r="D48" s="122"/>
+      <c r="E48" s="123"/>
+      <c r="F48" s="122"/>
+      <c r="G48" s="122"/>
+      <c r="H48" s="122"/>
+      <c r="I48" s="122"/>
+      <c r="J48" s="122"/>
+      <c r="K48" s="122"/>
+      <c r="L48" s="124"/>
+      <c r="M48" s="122"/>
+      <c r="N48" s="122"/>
+      <c r="O48" s="122"/>
+      <c r="P48" s="125" t="s">
         <v>170</v>
       </c>
-      <c r="Q48" s="129"/>
-      <c r="R48" s="129"/>
-      <c r="S48" s="129"/>
-      <c r="T48" s="129"/>
-      <c r="U48" s="133"/>
-      <c r="V48" s="134"/>
-      <c r="W48" s="133" t="s">
+      <c r="Q48" s="122"/>
+      <c r="R48" s="122"/>
+      <c r="S48" s="122"/>
+      <c r="T48" s="122"/>
+      <c r="U48" s="126"/>
+      <c r="V48" s="127"/>
+      <c r="W48" s="126" t="s">
         <v>171</v>
       </c>
-      <c r="X48" s="71"/>
-      <c r="Y48" s="71"/>
-      <c r="Z48" s="71"/>
-      <c r="AA48" s="71"/>
-      <c r="AB48" s="71"/>
-      <c r="AC48" s="71"/>
+      <c r="X48" s="65"/>
+      <c r="Y48" s="65"/>
+      <c r="Z48" s="65"/>
+      <c r="AA48" s="65"/>
+      <c r="AB48" s="65"/>
+      <c r="AC48" s="65"/>
     </row>
     <row r="49" spans="1:29" ht="66">
-      <c r="A49" s="135"/>
-      <c r="B49" s="136" t="s">
+      <c r="A49" s="128"/>
+      <c r="B49" s="129" t="s">
         <v>81</v>
       </c>
-      <c r="C49" s="137"/>
-      <c r="D49" s="137"/>
-      <c r="E49" s="138"/>
-      <c r="F49" s="97"/>
-      <c r="G49" s="97"/>
-      <c r="H49" s="97"/>
-      <c r="I49" s="97"/>
-      <c r="J49" s="97"/>
-      <c r="K49" s="97"/>
-      <c r="L49" s="71"/>
-      <c r="M49" s="97"/>
-      <c r="N49" s="139"/>
-      <c r="O49" s="97"/>
-      <c r="P49" s="140"/>
-      <c r="Q49" s="71"/>
-      <c r="R49" s="71"/>
-      <c r="S49" s="139" t="s">
+      <c r="C49" s="130"/>
+      <c r="D49" s="130"/>
+      <c r="E49" s="131"/>
+      <c r="F49" s="90"/>
+      <c r="G49" s="90"/>
+      <c r="H49" s="90"/>
+      <c r="I49" s="90"/>
+      <c r="J49" s="90"/>
+      <c r="K49" s="90"/>
+      <c r="L49" s="65"/>
+      <c r="M49" s="90"/>
+      <c r="N49" s="132"/>
+      <c r="O49" s="90"/>
+      <c r="P49" s="133"/>
+      <c r="Q49" s="65"/>
+      <c r="R49" s="65"/>
+      <c r="S49" s="132" t="s">
         <v>172</v>
       </c>
-      <c r="T49" s="71"/>
-      <c r="U49" s="141"/>
-      <c r="V49" s="141"/>
-      <c r="W49" s="141" t="s">
+      <c r="T49" s="65"/>
+      <c r="U49" s="134"/>
+      <c r="V49" s="134"/>
+      <c r="W49" s="134" t="s">
         <v>173</v>
       </c>
-      <c r="X49" s="71"/>
-      <c r="Y49" s="71"/>
-      <c r="Z49" s="71"/>
-      <c r="AA49" s="71"/>
-      <c r="AB49" s="71"/>
-      <c r="AC49" s="71"/>
+      <c r="X49" s="65"/>
+      <c r="Y49" s="65"/>
+      <c r="Z49" s="65"/>
+      <c r="AA49" s="65"/>
+      <c r="AB49" s="65"/>
+      <c r="AC49" s="65"/>
     </row>
     <row r="50" spans="1:29" ht="15" thickBot="1">
-      <c r="A50" s="142"/>
-      <c r="B50" s="143" t="s">
+      <c r="A50" s="135"/>
+      <c r="B50" s="136" t="s">
         <v>84</v>
       </c>
-      <c r="C50" s="144"/>
-      <c r="D50" s="144"/>
-      <c r="E50" s="145"/>
-      <c r="F50" s="146"/>
-      <c r="G50" s="146"/>
-      <c r="H50" s="146"/>
-      <c r="I50" s="146"/>
-      <c r="J50" s="146"/>
-      <c r="K50" s="146"/>
-      <c r="L50" s="146"/>
-      <c r="M50" s="146"/>
-      <c r="N50" s="146"/>
-      <c r="O50" s="146"/>
-      <c r="P50" s="147"/>
-      <c r="Q50" s="146"/>
-      <c r="R50" s="146"/>
-      <c r="S50" s="146"/>
-      <c r="T50" s="146"/>
-      <c r="U50" s="148"/>
-      <c r="V50" s="148"/>
-      <c r="W50" s="148"/>
-      <c r="X50" s="71"/>
-      <c r="Y50" s="71"/>
-      <c r="Z50" s="71"/>
-      <c r="AA50" s="71"/>
-      <c r="AB50" s="71"/>
-      <c r="AC50" s="71"/>
+      <c r="C50" s="137"/>
+      <c r="D50" s="137"/>
+      <c r="E50" s="138"/>
+      <c r="F50" s="139"/>
+      <c r="G50" s="139"/>
+      <c r="H50" s="139"/>
+      <c r="I50" s="139"/>
+      <c r="J50" s="139"/>
+      <c r="K50" s="139"/>
+      <c r="L50" s="139"/>
+      <c r="M50" s="139"/>
+      <c r="N50" s="139"/>
+      <c r="O50" s="139"/>
+      <c r="P50" s="140"/>
+      <c r="Q50" s="139"/>
+      <c r="R50" s="139"/>
+      <c r="S50" s="139"/>
+      <c r="T50" s="139"/>
+      <c r="U50" s="141"/>
+      <c r="V50" s="141"/>
+      <c r="W50" s="141"/>
+      <c r="X50" s="65"/>
+      <c r="Y50" s="65"/>
+      <c r="Z50" s="65"/>
+      <c r="AA50" s="65"/>
+      <c r="AB50" s="65"/>
+      <c r="AC50" s="65"/>
     </row>
     <row r="51" spans="1:29" ht="15" thickTop="1"/>
   </sheetData>
@@ -15925,11 +16160,11 @@
       <c r="I12" s="9"/>
     </row>
     <row r="15" spans="1:9" ht="21">
-      <c r="B15" s="64" t="s">
+      <c r="B15" s="142" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
+      <c r="C15" s="142"/>
+      <c r="D15" s="142"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="10" t="s">
@@ -16123,21 +16358,21 @@
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="148" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="69"/>
-      <c r="I8" s="69"/>
-      <c r="J8" s="69"/>
-      <c r="K8" s="69"/>
-      <c r="L8" s="69"/>
-      <c r="M8" s="69"/>
-      <c r="N8" s="69"/>
-      <c r="O8" s="69"/>
-      <c r="P8" s="69"/>
+      <c r="E8" s="148"/>
+      <c r="F8" s="148"/>
+      <c r="G8" s="148"/>
+      <c r="H8" s="148"/>
+      <c r="I8" s="148"/>
+      <c r="J8" s="148"/>
+      <c r="K8" s="148"/>
+      <c r="L8" s="148"/>
+      <c r="M8" s="148"/>
+      <c r="N8" s="148"/>
+      <c r="O8" s="148"/>
+      <c r="P8" s="148"/>
       <c r="Q8" s="11"/>
     </row>
     <row r="9" spans="1:18" ht="15.6">
@@ -17127,21 +17362,21 @@
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="148" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="69"/>
-      <c r="I8" s="69"/>
-      <c r="J8" s="69"/>
-      <c r="K8" s="69"/>
-      <c r="L8" s="69"/>
-      <c r="M8" s="69"/>
-      <c r="N8" s="69"/>
-      <c r="O8" s="69"/>
-      <c r="P8" s="69"/>
+      <c r="E8" s="148"/>
+      <c r="F8" s="148"/>
+      <c r="G8" s="148"/>
+      <c r="H8" s="148"/>
+      <c r="I8" s="148"/>
+      <c r="J8" s="148"/>
+      <c r="K8" s="148"/>
+      <c r="L8" s="148"/>
+      <c r="M8" s="148"/>
+      <c r="N8" s="148"/>
+      <c r="O8" s="148"/>
+      <c r="P8" s="148"/>
     </row>
     <row r="9" spans="1:16" ht="15.6">
       <c r="A9" s="11"/>

</xml_diff>

<commit_message>
checklist 1st week date updated
</commit_message>
<xml_diff>
--- a/ProjectManagement/Checklist.xlsx
+++ b/ProjectManagement/Checklist.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10112"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B585C7A-5B5C-144A-98D7-26BA12C84679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4282C8B0-6E26-7945-832C-3A61545264E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="25260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4880" yWindow="620" windowWidth="46320" windowHeight="25260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -1029,7 +1029,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1214,6 +1214,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9484,6 +9485,9 @@
       <c r="C15" s="65" t="s">
         <v>127</v>
       </c>
+      <c r="D15" s="70">
+        <v>45925</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
@@ -9494,8 +9498,11 @@
         <v>92</v>
       </c>
       <c r="C16" s="65"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D16" s="70">
+        <v>45927</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -9504,8 +9511,11 @@
         <v>93</v>
       </c>
       <c r="C17" s="65"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D17" s="70">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -9514,8 +9524,11 @@
         <v>4</v>
       </c>
       <c r="C18" s="65"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D18" s="70">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -9524,8 +9537,11 @@
         <v>5</v>
       </c>
       <c r="C19" s="65"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D19" s="70">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -9534,8 +9550,11 @@
         <v>7</v>
       </c>
       <c r="C20" s="65"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D20" s="70">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -9544,8 +9563,11 @@
         <v>94</v>
       </c>
       <c r="C21" s="65"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D21" s="70">
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -9554,8 +9576,11 @@
         <v>6</v>
       </c>
       <c r="C22" s="65"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D22" s="70">
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -9564,8 +9589,11 @@
         <v>8</v>
       </c>
       <c r="C23" s="65"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D23" s="70">
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -9574,8 +9602,11 @@
         <v>9</v>
       </c>
       <c r="C24" s="65"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D24" s="70">
+        <v>45957</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -9585,7 +9616,7 @@
       </c>
       <c r="C25" s="65"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -9597,7 +9628,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -9607,7 +9638,7 @@
       </c>
       <c r="C27" s="66"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -9617,7 +9648,7 @@
       </c>
       <c r="C28" s="66"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -9627,7 +9658,7 @@
       </c>
       <c r="C29" s="66"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -9637,7 +9668,7 @@
       </c>
       <c r="C30" s="66"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -9647,7 +9678,7 @@
       </c>
       <c r="C31" s="66"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>18</v>

</xml_diff>

<commit_message>
Project Management Document Plan Update
</commit_message>
<xml_diff>
--- a/ProjectManagement/Checklist.xlsx
+++ b/ProjectManagement/Checklist.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771B8B0B-7EAA-4E8E-AF94-455804FEBA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68133C3C-F1AB-422F-A3E8-7EA736020D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="164">
   <si>
     <t>Checklist</t>
   </si>
@@ -309,36 +309,6 @@
     <t>tests</t>
   </si>
   <si>
-    <t>1st Week</t>
-  </si>
-  <si>
-    <t>2nd week</t>
-  </si>
-  <si>
-    <t>3rd week</t>
-  </si>
-  <si>
-    <t>4th week</t>
-  </si>
-  <si>
-    <t>5th week</t>
-  </si>
-  <si>
-    <t>6th week</t>
-  </si>
-  <si>
-    <t>7th week</t>
-  </si>
-  <si>
-    <t>8th weeek</t>
-  </si>
-  <si>
-    <t>9th week</t>
-  </si>
-  <si>
-    <t>10 th weeek</t>
-  </si>
-  <si>
     <t>25.9.2025</t>
   </si>
   <si>
@@ -538,6 +508,24 @@
   </si>
   <si>
     <t>Professorenbesprechung- 15.12.2025</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>24.11.2025</t>
+  </si>
+  <si>
+    <t>7.12.2025</t>
+  </si>
+  <si>
+    <t>01.12.2025</t>
+  </si>
+  <si>
+    <t>14.12.2025</t>
+  </si>
+  <si>
+    <t>21.12.2025</t>
   </si>
 </sst>
 </file>
@@ -1351,24 +1339,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
@@ -1397,6 +1367,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2932,55 +2920,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>5862</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>58617</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>745951</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>104336</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="Rectangle 24">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC1A3FB7-5964-42B1-BA55-F2B4F07C6BAB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11519682" y="3807657"/>
-          <a:ext cx="740089" cy="45719"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-          </a:solidFill>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>298944</xdr:colOff>
       <xdr:row>32</xdr:row>
@@ -3014,6 +2953,349 @@
           <a:avLst>
             <a:gd name="adj" fmla="val 50000"/>
           </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="35" name="Rectangle 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5BC788C1-4FB7-42A6-8622-9BE4919A804D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11519682" y="3807657"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="36" name="Rectangle 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DEE6024D-8351-4937-A5C1-EF44533331CE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12312162" y="3990537"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="Rectangle 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EAB9B946-043F-47BA-8B39-E99219A76462}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13104642" y="4173417"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99C7855B-BB41-4E4B-A06E-2513BD2D63DF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="14689602" y="4722057"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="39" name="Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A25398F-FC21-46F3-9453-E817EA097DD3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13897122" y="4539177"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="Rectangle 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41BEDE30-C3DB-48C5-940F-953FED519DA1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="14689602" y="4904937"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="Rectangle 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44E7BD70-5B2F-4D27-B8B8-79015288E8D3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13104642" y="4356297"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
           <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
@@ -4643,6 +4925,300 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rectangle 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F53521E-9B23-4DDB-9AEF-5614DACB463C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11519682" y="3807657"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Rectangle 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF904BA2-04D3-4FE8-B8CF-66F508ACD0EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11519682" y="3807657"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7A56443-223D-4E27-A85B-9BAAA787B6FC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11519682" y="3807657"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Rectangle 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C535A4B-A0E4-4C3D-A859-1CE26AABCD4A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13897122" y="4356297"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13412D7B-DE19-4559-BEBC-BFCE59B67956}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13897122" y="4356297"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>5862</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>58617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>745951</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>104336</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Rectangle 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{586477E3-5420-4F43-8B6A-8D15A520A88E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13897122" y="4356297"/>
+          <a:ext cx="740089" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="008000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="17"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5071,11 +5647,12 @@
   <cols>
     <col min="1" max="1" width="15.77734375" customWidth="1"/>
     <col min="2" max="2" width="55" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -5084,7 +5661,7 @@
         <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="2" t="s">
@@ -5096,7 +5673,7 @@
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="65">
+      <c r="B5" s="59">
         <v>7026787</v>
       </c>
       <c r="H5" s="5" t="s">
@@ -5113,11 +5690,11 @@
       <c r="I6" s="9"/>
     </row>
     <row r="9" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -5139,12 +5716,12 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
+      <c r="B14" s="69"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -5153,11 +5730,9 @@
       <c r="B15" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="60" t="s">
+      <c r="C15" s="70"/>
+      <c r="D15" s="58" t="s">
         <v>91</v>
-      </c>
-      <c r="D15" s="58" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -5168,9 +5743,9 @@
       <c r="B16" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="60"/>
+      <c r="C16" s="70"/>
       <c r="D16" s="58" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -5181,9 +5756,9 @@
       <c r="B17" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="60"/>
+      <c r="C17" s="70"/>
       <c r="D17" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -5194,9 +5769,9 @@
       <c r="B18" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="60"/>
+      <c r="C18" s="70"/>
       <c r="D18" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -5207,9 +5782,9 @@
       <c r="B19" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="60"/>
+      <c r="C19" s="70"/>
       <c r="D19" s="58" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -5220,9 +5795,9 @@
       <c r="B20" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="60"/>
+      <c r="C20" s="70"/>
       <c r="D20" s="58" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -5233,9 +5808,9 @@
       <c r="B21" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="60"/>
+      <c r="C21" s="70"/>
       <c r="D21" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -5246,9 +5821,9 @@
       <c r="B22" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="60"/>
+      <c r="C22" s="70"/>
       <c r="D22" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -5259,9 +5834,9 @@
       <c r="B23" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="60"/>
+      <c r="C23" s="70"/>
       <c r="D23" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -5272,9 +5847,9 @@
       <c r="B24" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="60"/>
+      <c r="C24" s="70"/>
       <c r="D24" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -5285,9 +5860,9 @@
       <c r="B25" s="55" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="60"/>
+      <c r="C25" s="70"/>
       <c r="D25" s="58" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -5298,11 +5873,9 @@
       <c r="B26" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="61" t="s">
-        <v>92</v>
-      </c>
+      <c r="C26" s="71"/>
       <c r="D26" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -5313,9 +5886,9 @@
       <c r="B27" t="s">
         <v>12</v>
       </c>
-      <c r="C27" s="61"/>
+      <c r="C27" s="71"/>
       <c r="D27" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -5326,9 +5899,9 @@
       <c r="B28" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="61"/>
+      <c r="C28" s="71"/>
       <c r="D28" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -5339,9 +5912,9 @@
       <c r="B29" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="61"/>
+      <c r="C29" s="71"/>
       <c r="D29" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -5352,9 +5925,9 @@
       <c r="B30" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="61"/>
+      <c r="C30" s="71"/>
       <c r="D30" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -5365,9 +5938,9 @@
       <c r="B31" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="61"/>
+      <c r="C31" s="71"/>
       <c r="D31" s="57" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -5378,9 +5951,9 @@
       <c r="B32" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="61"/>
+      <c r="C32" s="71"/>
       <c r="D32" s="57" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -5391,9 +5964,9 @@
       <c r="B33" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="61"/>
+      <c r="C33" s="71"/>
       <c r="D33" s="57" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -5404,11 +5977,9 @@
       <c r="B34" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="60" t="s">
-        <v>93</v>
-      </c>
+      <c r="C34" s="70"/>
       <c r="D34" s="57" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -5419,9 +5990,9 @@
       <c r="B35" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="60"/>
+      <c r="C35" s="70"/>
       <c r="D35" s="57" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -5432,9 +6003,9 @@
       <c r="B36" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="C36" s="60"/>
+      <c r="C36" s="70"/>
       <c r="D36" s="57" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -5445,18 +6016,18 @@
       <c r="B37" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="C37" s="60"/>
+      <c r="C37" s="70"/>
       <c r="D37" s="57" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A38" s="59" t="s">
+      <c r="A38" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="59"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
+      <c r="B38" s="69"/>
+      <c r="C38" s="69"/>
+      <c r="D38" s="69"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
@@ -5466,11 +6037,9 @@
       <c r="B39" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="61" t="s">
-        <v>94</v>
-      </c>
+      <c r="C39" s="71"/>
       <c r="D39" s="57" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -5481,9 +6050,9 @@
       <c r="B40" t="s">
         <v>28</v>
       </c>
-      <c r="C40" s="61"/>
+      <c r="C40" s="71"/>
       <c r="D40" s="57" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -5494,9 +6063,9 @@
       <c r="B41" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="61"/>
+      <c r="C41" s="71"/>
       <c r="D41" s="57" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
@@ -5507,9 +6076,9 @@
       <c r="B42" t="s">
         <v>38</v>
       </c>
-      <c r="C42" s="61"/>
+      <c r="C42" s="71"/>
       <c r="D42" s="57" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
@@ -5520,9 +6089,9 @@
       <c r="B43" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="61"/>
+      <c r="C43" s="71"/>
       <c r="D43" s="57" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
@@ -5533,9 +6102,9 @@
       <c r="B44" t="s">
         <v>85</v>
       </c>
-      <c r="C44" s="61"/>
+      <c r="C44" s="71"/>
       <c r="D44" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
@@ -5546,9 +6115,9 @@
       <c r="B45" t="s">
         <v>84</v>
       </c>
-      <c r="C45" s="61"/>
+      <c r="C45" s="71"/>
       <c r="D45" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -5559,11 +6128,9 @@
       <c r="B46" s="55" t="s">
         <v>70</v>
       </c>
-      <c r="C46" s="62" t="s">
-        <v>95</v>
-      </c>
+      <c r="C46" s="72"/>
       <c r="D46" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
@@ -5574,9 +6141,9 @@
       <c r="B47" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="62"/>
+      <c r="C47" s="72"/>
       <c r="D47" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
@@ -5587,9 +6154,9 @@
       <c r="B48" s="55" t="s">
         <v>72</v>
       </c>
-      <c r="C48" s="62"/>
+      <c r="C48" s="72"/>
       <c r="D48" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -5600,9 +6167,9 @@
       <c r="B49" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="C49" s="62"/>
+      <c r="C49" s="72"/>
       <c r="D49" s="57" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
@@ -5613,11 +6180,9 @@
       <c r="B50" t="s">
         <v>74</v>
       </c>
-      <c r="C50" s="63" t="s">
-        <v>96</v>
-      </c>
+      <c r="C50" s="73"/>
       <c r="D50" s="57" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
@@ -5628,9 +6193,9 @@
       <c r="B51" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="63"/>
+      <c r="C51" s="73"/>
       <c r="D51" s="57" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
@@ -5641,9 +6206,9 @@
       <c r="B52" t="s">
         <v>86</v>
       </c>
-      <c r="C52" s="63"/>
+      <c r="C52" s="73"/>
       <c r="D52" s="57" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
@@ -5655,11 +6220,9 @@
         <f>[1]Report!$A$207</f>
         <v>Homework "Literature"</v>
       </c>
-      <c r="C53" s="62" t="s">
-        <v>97</v>
-      </c>
+      <c r="C53" s="72"/>
       <c r="D53" s="57" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
@@ -5670,9 +6233,9 @@
       <c r="B54" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="C54" s="62"/>
+      <c r="C54" s="72"/>
       <c r="D54" s="57" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -5683,9 +6246,9 @@
       <c r="B55" s="55" t="s">
         <v>80</v>
       </c>
-      <c r="C55" s="62"/>
+      <c r="C55" s="72"/>
       <c r="D55" s="57" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
@@ -5696,11 +6259,9 @@
       <c r="B56" t="s">
         <v>79</v>
       </c>
-      <c r="C56" s="63" t="s">
-        <v>98</v>
-      </c>
+      <c r="C56" s="73"/>
       <c r="D56" s="57" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -5711,9 +6272,9 @@
       <c r="B57" t="s">
         <v>81</v>
       </c>
-      <c r="C57" s="63"/>
+      <c r="C57" s="73"/>
       <c r="D57" s="57" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -5724,9 +6285,9 @@
       <c r="B58" t="s">
         <v>77</v>
       </c>
-      <c r="C58" s="63"/>
+      <c r="C58" s="73"/>
       <c r="D58" s="57" t="s">
-        <v>110</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -5737,9 +6298,9 @@
       <c r="B59" t="s">
         <v>78</v>
       </c>
-      <c r="C59" s="63"/>
+      <c r="C59" s="73"/>
       <c r="D59" s="57" t="s">
-        <v>110</v>
+        <v>161</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -5750,8 +6311,9 @@
       <c r="B60" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="C60" s="62" t="s">
-        <v>99</v>
+      <c r="C60" s="72"/>
+      <c r="D60" s="57" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
@@ -5762,7 +6324,10 @@
       <c r="B61" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="C61" s="62"/>
+      <c r="C61" s="72"/>
+      <c r="D61" s="57" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
@@ -5772,7 +6337,10 @@
       <c r="B62" s="55" t="s">
         <v>88</v>
       </c>
-      <c r="C62" s="62"/>
+      <c r="C62" s="72"/>
+      <c r="D62" s="57" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
@@ -5782,8 +6350,9 @@
       <c r="B63" t="s">
         <v>87</v>
       </c>
-      <c r="C63" s="63" t="s">
-        <v>100</v>
+      <c r="C63" s="73"/>
+      <c r="D63" s="57" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
@@ -5794,7 +6363,10 @@
       <c r="B64" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="C64" s="63"/>
+      <c r="C64" s="73"/>
+      <c r="D64" s="57" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65">
@@ -5804,15 +6376,18 @@
       <c r="B65" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="C65" s="63"/>
+      <c r="C65" s="73"/>
+      <c r="D65" s="57" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="66" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A66" s="59" t="s">
+      <c r="A66" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="B66" s="59"/>
-      <c r="C66" s="59"/>
-      <c r="D66" s="59"/>
+      <c r="B66" s="69"/>
+      <c r="C66" s="69"/>
+      <c r="D66" s="69"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67">
@@ -6061,21 +6636,21 @@
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="64" t="s">
-        <v>161</v>
-      </c>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64"/>
-      <c r="G8" s="64"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="64"/>
-      <c r="M8" s="64"/>
-      <c r="N8" s="64"/>
-      <c r="O8" s="64"/>
-      <c r="P8" s="64"/>
+      <c r="D8" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="74"/>
+      <c r="K8" s="74"/>
+      <c r="L8" s="74"/>
+      <c r="M8" s="74"/>
+      <c r="N8" s="74"/>
+      <c r="O8" s="74"/>
+      <c r="P8" s="74"/>
     </row>
     <row r="9" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="11"/>
@@ -6113,11 +6688,11 @@
     </row>
     <row r="11" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="74" t="s">
-        <v>162</v>
-      </c>
-      <c r="D11" s="70">
+      <c r="B11" s="61"/>
+      <c r="C11" s="68" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="64">
         <v>40</v>
       </c>
       <c r="E11" s="15">
@@ -6159,11 +6734,11 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="16"/>
-      <c r="B12" s="68"/>
-      <c r="C12" s="74" t="s">
-        <v>163</v>
-      </c>
-      <c r="D12" s="71">
+      <c r="B12" s="62"/>
+      <c r="C12" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="D12" s="65">
         <v>1</v>
       </c>
       <c r="E12" s="19">
@@ -6207,13 +6782,13 @@
       <c r="A13" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="69" t="s">
-        <v>164</v>
-      </c>
-      <c r="C13" s="74" t="s">
+      <c r="B13" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="C13" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="72"/>
+      <c r="D13" s="66"/>
       <c r="E13" s="25"/>
       <c r="F13" s="25"/>
       <c r="G13" s="25"/>
@@ -6232,9 +6807,9 @@
         <v>1</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>145</v>
-      </c>
-      <c r="C14" s="73">
+        <v>135</v>
+      </c>
+      <c r="C14" s="67">
         <v>1</v>
       </c>
       <c r="D14" s="30"/>
@@ -6257,7 +6832,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C15" s="35">
         <v>1</v>
@@ -6282,7 +6857,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="34" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C16" s="35">
         <v>2</v>
@@ -6307,7 +6882,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="34" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C17" s="35">
         <v>3</v>
@@ -6332,7 +6907,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C18" s="35">
         <v>4</v>
@@ -6357,7 +6932,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="34" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C19" s="35">
         <v>5</v>
@@ -6382,7 +6957,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="34" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C20" s="35">
         <v>5</v>
@@ -6407,7 +6982,7 @@
         <v>8</v>
       </c>
       <c r="B21" s="34" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C21" s="35">
         <v>6</v>
@@ -6432,7 +7007,7 @@
         <v>9</v>
       </c>
       <c r="B22" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="C22" s="35">
         <v>7</v>
@@ -6457,7 +7032,7 @@
         <v>10</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C23" s="35">
         <v>8</v>
@@ -6482,7 +7057,7 @@
         <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="C24" s="35">
         <v>9</v>
@@ -6507,7 +7082,7 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C25" s="35">
         <v>10</v>
@@ -6532,7 +7107,7 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C26" s="35">
         <v>11</v>
@@ -6547,7 +7122,9 @@
       <c r="K26" s="37"/>
       <c r="L26" s="37"/>
       <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
+      <c r="N26" s="37" t="s">
+        <v>158</v>
+      </c>
       <c r="O26" s="37"/>
       <c r="P26" s="38"/>
     </row>
@@ -6557,7 +7134,7 @@
         <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="C27" s="35">
         <v>12</v>
@@ -6582,7 +7159,7 @@
         <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C28" s="35">
         <v>13</v>
@@ -6652,7 +7229,7 @@
       <c r="N31" s="49"/>
       <c r="O31" s="49"/>
       <c r="P31" s="11" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
@@ -6660,7 +7237,7 @@
       <c r="B32" s="34"/>
       <c r="C32" s="35"/>
       <c r="D32" s="36" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E32" s="37"/>
       <c r="F32" s="37"/>
@@ -6674,7 +7251,7 @@
       <c r="N32" s="37"/>
       <c r="O32" s="51"/>
       <c r="P32" s="36" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="53.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -6682,38 +7259,38 @@
       <c r="B33" s="40"/>
       <c r="C33" s="41"/>
       <c r="D33" s="42"/>
-      <c r="E33" s="66" t="s">
-        <v>132</v>
-      </c>
-      <c r="F33" s="66" t="s">
-        <v>133</v>
-      </c>
-      <c r="G33" s="66" t="s">
+      <c r="E33" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="F33" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="G33" s="60" t="s">
+        <v>124</v>
+      </c>
+      <c r="H33" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="H33" s="66" t="s">
-        <v>135</v>
-      </c>
-      <c r="I33" s="66" t="s">
-        <v>144</v>
-      </c>
-      <c r="J33" s="66" t="s">
-        <v>165</v>
-      </c>
-      <c r="K33" s="66" t="s">
-        <v>141</v>
-      </c>
-      <c r="L33" s="66" t="s">
-        <v>140</v>
-      </c>
-      <c r="M33" s="66" t="s">
-        <v>166</v>
-      </c>
-      <c r="N33" s="66" t="s">
-        <v>139</v>
-      </c>
-      <c r="O33" s="66" t="s">
-        <v>167</v>
+      <c r="J33" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="K33" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="L33" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="M33" s="60" t="s">
+        <v>156</v>
+      </c>
+      <c r="N33" s="60" t="s">
+        <v>129</v>
+      </c>
+      <c r="O33" s="60" t="s">
+        <v>157</v>
       </c>
       <c r="P33" s="43"/>
     </row>
@@ -7002,21 +7579,21 @@
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="64" t="s">
-        <v>111</v>
-      </c>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64"/>
-      <c r="G8" s="64"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="64"/>
-      <c r="M8" s="64"/>
-      <c r="N8" s="64"/>
-      <c r="O8" s="64"/>
-      <c r="P8" s="64"/>
+      <c r="D8" s="74" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="74"/>
+      <c r="K8" s="74"/>
+      <c r="L8" s="74"/>
+      <c r="M8" s="74"/>
+      <c r="N8" s="74"/>
+      <c r="O8" s="74"/>
+      <c r="P8" s="74"/>
     </row>
     <row r="9" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="11"/>
@@ -7173,7 +7750,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C14" s="29">
         <v>1</v>
@@ -7198,7 +7775,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="34" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C15" s="35">
         <v>1</v>
@@ -7223,7 +7800,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="34" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C16" s="35">
         <v>2</v>
@@ -7248,7 +7825,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="34" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C17" s="35">
         <v>3</v>
@@ -7273,7 +7850,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C18" s="35">
         <v>4</v>
@@ -7298,7 +7875,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="34" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C19" s="35">
         <v>5</v>
@@ -7323,7 +7900,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="34" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C20" s="35">
         <v>5</v>
@@ -7348,7 +7925,7 @@
         <v>8</v>
       </c>
       <c r="B21" s="34" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C21" s="35">
         <v>6</v>
@@ -7373,7 +7950,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="34" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C22" s="35">
         <v>7</v>
@@ -7398,7 +7975,7 @@
         <v>10</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C23" s="35">
         <v>8</v>
@@ -7423,7 +8000,7 @@
         <v>11</v>
       </c>
       <c r="B24" s="34" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C24" s="35">
         <v>9</v>
@@ -7448,7 +8025,7 @@
         <v>12</v>
       </c>
       <c r="B25" s="34" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C25" s="35">
         <v>10</v>
@@ -7473,7 +8050,7 @@
         <v>13</v>
       </c>
       <c r="B26" s="34" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C26" s="35">
         <v>11</v>
@@ -7488,7 +8065,9 @@
       <c r="K26" s="37"/>
       <c r="L26" s="37"/>
       <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
+      <c r="N26" s="37" t="s">
+        <v>158</v>
+      </c>
       <c r="O26" s="37"/>
       <c r="P26" s="38"/>
     </row>
@@ -7498,7 +8077,7 @@
         <v>14</v>
       </c>
       <c r="B27" s="34" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C27" s="35">
         <v>12</v>
@@ -7523,7 +8102,7 @@
         <v>15</v>
       </c>
       <c r="B28" s="34" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C28" s="35">
         <v>13</v>
@@ -7595,7 +8174,7 @@
       <c r="N31" s="49"/>
       <c r="O31" s="49"/>
       <c r="P31" s="50" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
@@ -7605,7 +8184,7 @@
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="36" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E32" s="37"/>
       <c r="F32" s="37"/>
@@ -7619,7 +8198,7 @@
       <c r="N32" s="37"/>
       <c r="O32" s="51"/>
       <c r="P32" s="36" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
@@ -7629,38 +8208,38 @@
       </c>
       <c r="C33" s="41"/>
       <c r="D33" s="42"/>
-      <c r="E33" s="66" t="s">
+      <c r="E33" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="F33" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="G33" s="60" t="s">
+        <v>124</v>
+      </c>
+      <c r="H33" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="60" t="s">
+        <v>134</v>
+      </c>
+      <c r="J33" s="60" t="s">
         <v>132</v>
       </c>
-      <c r="F33" s="66" t="s">
-        <v>133</v>
-      </c>
-      <c r="G33" s="66" t="s">
-        <v>134</v>
-      </c>
-      <c r="H33" s="66" t="s">
-        <v>135</v>
-      </c>
-      <c r="I33" s="66" t="s">
-        <v>144</v>
-      </c>
-      <c r="J33" s="66" t="s">
-        <v>142</v>
-      </c>
-      <c r="K33" s="66" t="s">
-        <v>141</v>
-      </c>
-      <c r="L33" s="66" t="s">
-        <v>140</v>
-      </c>
-      <c r="M33" s="66" t="s">
-        <v>138</v>
-      </c>
-      <c r="N33" s="66" t="s">
-        <v>139</v>
-      </c>
-      <c r="O33" s="66" t="s">
-        <v>137</v>
+      <c r="K33" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="L33" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="M33" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="N33" s="60" t="s">
+        <v>129</v>
+      </c>
+      <c r="O33" s="60" t="s">
+        <v>127</v>
       </c>
       <c r="P33" s="43"/>
     </row>
@@ -7831,16 +8410,16 @@
   <sheetData>
     <row r="7" spans="1:9" ht="23.4" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="2" t="s">
@@ -7869,11 +8448,11 @@
       <c r="I12" s="9"/>
     </row>
     <row r="15" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">

</xml_diff>